<commit_message>
Finishing plotting the other sites for tile issues
</commit_message>
<xml_diff>
--- a/data/veg (raw).xlsx
+++ b/data/veg (raw).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1234" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{480FAB72-8786-4F73-B863-1B94BAD03463}"/>
+  <xr:revisionPtr revIDLastSave="1289" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5429A239-3AA6-4F7B-A708-396DBE4B2016}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
+    <workbookView minimized="1" xWindow="2844" yWindow="1140" windowWidth="9996" windowHeight="6912" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
   </bookViews>
   <sheets>
     <sheet name="winter" sheetId="1" r:id="rId1"/>
@@ -557,7 +557,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -746,6 +746,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -983,7 +989,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1020,11 +1026,10 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="18" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1407,6 +1412,7 @@
   <dimension ref="A1:W196"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="6" max="6" width="18.33203125" customWidth="1"/>
     <col min="9" max="9" width="12.77734375" customWidth="1"/>
     <col min="10" max="10" width="11.6640625" customWidth="1"/>
     <col min="21" max="21" width="14.5546875" customWidth="1"/>
@@ -1634,8 +1640,8 @@
         <v>46074</v>
       </c>
       <c r="G4" s="12">
-        <f>SUM(H2:H4)</f>
-        <v>100</v>
+        <f>SUM(H2:H3)</f>
+        <v>70</v>
       </c>
       <c r="H4" s="12">
         <v>30</v>
@@ -4029,53 +4035,53 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A60" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B60" t="s">
-        <v>24</v>
-      </c>
-      <c r="C60" t="s">
+    <row r="60" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B60" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C60" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="31">
         <v>1</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="31">
         <v>0.5</v>
       </c>
-      <c r="F60" s="9">
+      <c r="F60" s="32">
         <v>46073</v>
       </c>
-      <c r="H60">
+      <c r="H60" s="31">
         <v>60</v>
       </c>
-      <c r="I60" t="s">
+      <c r="I60" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="J60">
+      <c r="J60" s="31">
         <v>15</v>
       </c>
-      <c r="K60" t="s">
+      <c r="K60" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L60">
+      <c r="L60" s="31">
         <v>18</v>
       </c>
-      <c r="N60">
+      <c r="N60" s="31">
         <v>13</v>
       </c>
-      <c r="P60">
+      <c r="P60" s="31">
         <v>10</v>
       </c>
-      <c r="R60">
+      <c r="R60" s="31">
         <v>20.5</v>
       </c>
-      <c r="T60">
+      <c r="T60" s="31">
         <v>20.5</v>
       </c>
-      <c r="V60" s="16">
+      <c r="V60" s="33">
         <v>0.43958333333333333</v>
       </c>
     </row>
@@ -4212,68 +4218,68 @@
         <v>87</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A64" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B64" t="s">
-        <v>24</v>
-      </c>
-      <c r="C64" t="s">
+    <row r="64" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B64" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C64" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="31">
         <v>1</v>
       </c>
-      <c r="E64">
-        <v>2</v>
-      </c>
-      <c r="F64" s="9">
+      <c r="E64" s="31">
+        <v>2</v>
+      </c>
+      <c r="F64" s="32">
         <v>46073</v>
       </c>
-      <c r="H64">
+      <c r="H64" s="31">
         <v>50</v>
       </c>
-      <c r="I64" t="s">
-        <v>28</v>
-      </c>
-      <c r="J64">
+      <c r="I64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="J64" s="31">
         <v>29</v>
       </c>
-      <c r="K64" t="s">
-        <v>28</v>
-      </c>
-      <c r="L64">
+      <c r="K64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="L64" s="31">
         <v>31</v>
       </c>
-      <c r="M64" t="s">
-        <v>28</v>
-      </c>
-      <c r="N64">
+      <c r="M64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="N64" s="31">
         <v>29</v>
       </c>
-      <c r="O64" t="s">
-        <v>28</v>
-      </c>
-      <c r="P64">
-        <v>28</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>28</v>
-      </c>
-      <c r="R64">
+      <c r="O64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="P64" s="31">
+        <v>28</v>
+      </c>
+      <c r="Q64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="R64" s="31">
         <v>27.5</v>
       </c>
-      <c r="S64" t="s">
-        <v>28</v>
-      </c>
-      <c r="T64">
+      <c r="S64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="T64" s="31">
         <v>31</v>
       </c>
-      <c r="U64" t="s">
-        <v>28</v>
-      </c>
-      <c r="V64" s="16">
+      <c r="U64" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="V64" s="33">
         <v>0.45347222222222222</v>
       </c>
     </row>
@@ -6082,7 +6088,7 @@
       <c r="T104">
         <v>35</v>
       </c>
-      <c r="V104" s="30" t="s">
+      <c r="V104" s="25" t="s">
         <v>102</v>
       </c>
     </row>
@@ -10421,8 +10427,8 @@
         <v>46184</v>
       </c>
       <c r="G4" s="12">
-        <f>SUM(H2:H4)</f>
-        <v>100</v>
+        <f>SUM(H2:H3)</f>
+        <v>75</v>
       </c>
       <c r="H4" s="12">
         <v>25</v>
@@ -10557,8 +10563,8 @@
         <v>46184</v>
       </c>
       <c r="G7" s="12">
-        <f>SUM(H5:H7)</f>
-        <v>100</v>
+        <f>SUM(H5:H6)</f>
+        <v>65</v>
       </c>
       <c r="H7" s="12">
         <v>35</v>
@@ -10696,8 +10702,8 @@
         <v>46184</v>
       </c>
       <c r="G10" s="12">
-        <f>SUM(H8:H10)</f>
-        <v>100</v>
+        <f>SUM(H8:H9)</f>
+        <v>95</v>
       </c>
       <c r="H10" s="12">
         <v>5</v>
@@ -10799,8 +10805,8 @@
         <v>46184</v>
       </c>
       <c r="G13" s="12">
-        <f>SUM(H11:H13)</f>
-        <v>105</v>
+        <f>SUM(H12:H13)</f>
+        <v>95</v>
       </c>
       <c r="H13" s="14">
         <v>90</v>
@@ -11100,8 +11106,8 @@
         <v>46184</v>
       </c>
       <c r="G19" s="12">
-        <f>SUM(H14:H19)</f>
-        <v>115</v>
+        <f>SUM(H14:H17, H19)</f>
+        <v>105</v>
       </c>
       <c r="H19" s="12">
         <v>10</v>
@@ -11344,8 +11350,8 @@
         <v>46184</v>
       </c>
       <c r="G25" s="12">
-        <f>SUM(H20:H25)</f>
-        <v>170</v>
+        <f>SUM(H20:H23, H25)</f>
+        <v>140</v>
       </c>
       <c r="H25" s="14">
         <v>40</v>
@@ -11534,8 +11540,8 @@
         <v>46184</v>
       </c>
       <c r="G29" s="12">
-        <f>SUM(H26:H29)</f>
-        <v>105</v>
+        <f>SUM(H26:H27, H29)</f>
+        <v>100</v>
       </c>
       <c r="H29" s="12">
         <v>10</v>
@@ -11887,8 +11893,8 @@
         <v>46184</v>
       </c>
       <c r="G37" s="12">
-        <f>SUM(H34:H37)</f>
-        <v>110</v>
+        <f>SUM(H34:H36)</f>
+        <v>105</v>
       </c>
       <c r="H37" s="12">
         <v>5</v>
@@ -12195,8 +12201,8 @@
         <v>46184</v>
       </c>
       <c r="G44" s="12">
-        <f>SUM(H41:H44)</f>
-        <v>100</v>
+        <f>SUM(H41:H43)</f>
+        <v>95</v>
       </c>
       <c r="H44" s="12">
         <v>5</v>
@@ -12554,8 +12560,8 @@
         <v>46184</v>
       </c>
       <c r="G52" s="12">
-        <f>SUM(H49:H52)</f>
-        <v>110</v>
+        <f>SUM(H49:H51)</f>
+        <v>105</v>
       </c>
       <c r="H52" s="12">
         <v>5</v>
@@ -12723,8 +12729,8 @@
         <v>46184</v>
       </c>
       <c r="G56" s="12">
-        <f>SUM(H53:H56)</f>
-        <v>125</v>
+        <f>SUM(H53:H55)</f>
+        <v>115</v>
       </c>
       <c r="H56" s="12">
         <v>10</v>
@@ -13022,8 +13028,8 @@
         <v>46182</v>
       </c>
       <c r="G62" s="12">
-        <f>SUM(H60:H62)</f>
-        <v>100</v>
+        <f>SUM(H60:H61)</f>
+        <v>90</v>
       </c>
       <c r="H62" s="12">
         <v>10</v>
@@ -13125,8 +13131,8 @@
         <v>46182</v>
       </c>
       <c r="G64" s="12">
-        <f>SUM(H63:H64)</f>
-        <v>100</v>
+        <f>SUM(H63)</f>
+        <v>85</v>
       </c>
       <c r="H64" s="12">
         <v>15</v>
@@ -13228,8 +13234,8 @@
         <v>46182</v>
       </c>
       <c r="G66">
-        <f>SUM(H65:H66)</f>
-        <v>120</v>
+        <f>SUM(H65)</f>
+        <v>80</v>
       </c>
       <c r="H66">
         <v>40</v>
@@ -13331,8 +13337,8 @@
         <v>46182</v>
       </c>
       <c r="G68" s="12">
-        <f>SUM(H67:H68)</f>
-        <v>100</v>
+        <f>SUM(H67)</f>
+        <v>90</v>
       </c>
       <c r="H68" s="12">
         <v>10</v>
@@ -13467,8 +13473,8 @@
         <v>46182</v>
       </c>
       <c r="G71" s="12">
-        <f>SUM(H69:H71)</f>
-        <v>110</v>
+        <f>SUM(H70:H71)</f>
+        <v>105</v>
       </c>
       <c r="H71" s="12">
         <v>55</v>
@@ -13705,8 +13711,8 @@
         <v>46182</v>
       </c>
       <c r="G76" s="12">
-        <f>SUM(H72:H76)</f>
-        <v>155</v>
+        <f>SUM(H72:H75)</f>
+        <v>150</v>
       </c>
       <c r="H76" s="12">
         <v>5</v>
@@ -13742,7 +13748,7 @@
         <v>46182</v>
       </c>
       <c r="G77" s="19">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H77" s="19">
         <v>15</v>
@@ -13862,8 +13868,8 @@
         <v>46182</v>
       </c>
       <c r="G80" s="12">
-        <f>SUM(H78:H80)</f>
-        <v>105</v>
+        <f>SUM(H78, H80)</f>
+        <v>100</v>
       </c>
       <c r="H80" s="14">
         <v>80</v>
@@ -13989,8 +13995,8 @@
         <v>46182</v>
       </c>
       <c r="G82" s="12">
-        <f>SUM(H81:H82)</f>
-        <v>100</v>
+        <f>SUM(H81)</f>
+        <v>85</v>
       </c>
       <c r="H82" s="12">
         <v>15</v>
@@ -14122,8 +14128,8 @@
         <v>46182</v>
       </c>
       <c r="G85" s="12">
-        <f>SUM(H83:H85)</f>
-        <v>135</v>
+        <f>SUM(H83:H84)</f>
+        <v>130</v>
       </c>
       <c r="H85" s="12">
         <v>5</v>
@@ -14225,8 +14231,8 @@
         <v>46182</v>
       </c>
       <c r="G87" s="12">
-        <f>SUM(H86:H87)</f>
-        <v>100</v>
+        <f>SUM(H86)</f>
+        <v>90</v>
       </c>
       <c r="H87" s="12">
         <v>10</v>
@@ -14328,8 +14334,8 @@
         <v>46182</v>
       </c>
       <c r="G89" s="12">
-        <f>SUM(H88:H89)</f>
-        <v>100</v>
+        <f>SUM(H88)</f>
+        <v>95</v>
       </c>
       <c r="H89" s="12">
         <v>5</v>
@@ -14411,40 +14417,40 @@
         <v>0.45833333333333331</v>
       </c>
     </row>
-    <row r="91" spans="1:23" s="31" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B91" s="31" t="s">
+      <c r="B91" t="s">
         <v>73</v>
       </c>
-      <c r="C91" s="31" t="s">
+      <c r="C91" t="s">
         <v>41</v>
       </c>
-      <c r="D91" s="31">
-        <v>2</v>
-      </c>
-      <c r="E91" s="31">
+      <c r="D91">
+        <v>2</v>
+      </c>
+      <c r="E91">
         <v>48</v>
       </c>
-      <c r="F91" s="32">
+      <c r="F91" s="9">
         <v>46182</v>
       </c>
-      <c r="G91" s="31">
-        <f>SUM(H90:H91)</f>
-        <v>100</v>
-      </c>
-      <c r="H91" s="31">
+      <c r="G91">
+        <f>SUM(H90)</f>
+        <v>95</v>
+      </c>
+      <c r="H91">
         <v>5</v>
       </c>
-      <c r="I91" s="31" t="s">
+      <c r="I91" t="s">
         <v>29</v>
       </c>
-      <c r="J91" s="31" t="e">
+      <c r="J91" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T91" s="31">
+      <c r="T91">
         <v>0</v>
       </c>
     </row>
@@ -14472,49 +14478,49 @@
         <v>31</v>
       </c>
     </row>
-    <row r="93" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A93" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B93" s="31" t="s">
+      <c r="B93" t="s">
         <v>73</v>
       </c>
-      <c r="C93" s="31" t="s">
+      <c r="C93" t="s">
         <v>52</v>
       </c>
-      <c r="D93" s="31">
+      <c r="D93">
         <v>1</v>
       </c>
-      <c r="E93" s="31">
+      <c r="E93">
         <v>0.5</v>
       </c>
-      <c r="F93" s="32"/>
-      <c r="H93" s="31">
+      <c r="F93" s="9"/>
+      <c r="H93">
         <v>80</v>
       </c>
-      <c r="I93" s="31" t="s">
+      <c r="I93" t="s">
         <v>36</v>
       </c>
-      <c r="J93" s="31">
+      <c r="J93">
         <f>AVERAGE(L93, N93, P93, R93)</f>
         <v>14.5</v>
       </c>
-      <c r="K93" s="31" t="s">
+      <c r="K93" t="s">
         <v>36</v>
       </c>
-      <c r="L93" s="31">
+      <c r="L93">
         <v>13.5</v>
       </c>
-      <c r="N93" s="31">
+      <c r="N93">
         <v>13</v>
       </c>
-      <c r="P93" s="31">
+      <c r="P93">
         <v>15</v>
       </c>
-      <c r="R93" s="31">
+      <c r="R93">
         <v>16.5</v>
       </c>
-      <c r="T93" s="31">
+      <c r="T93">
         <v>16.5</v>
       </c>
     </row>
@@ -14604,46 +14610,46 @@
         <v>22</v>
       </c>
     </row>
-    <row r="96" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A96" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B96" s="31" t="s">
+      <c r="B96" t="s">
         <v>73</v>
       </c>
-      <c r="C96" s="31" t="s">
+      <c r="C96" t="s">
         <v>52</v>
       </c>
-      <c r="D96" s="31">
+      <c r="D96">
         <v>1</v>
       </c>
-      <c r="E96" s="31">
-        <v>2</v>
-      </c>
-      <c r="F96" s="32"/>
-      <c r="H96" s="31">
+      <c r="E96">
+        <v>2</v>
+      </c>
+      <c r="F96" s="9"/>
+      <c r="H96">
         <v>10</v>
       </c>
-      <c r="I96" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J96" s="31">
+      <c r="I96" t="s">
+        <v>28</v>
+      </c>
+      <c r="J96">
         <f>AVERAGE(L96, N96, P96, R96)</f>
         <v>33</v>
       </c>
-      <c r="L96" s="31">
+      <c r="L96">
         <v>31</v>
       </c>
-      <c r="N96" s="31" t="s">
+      <c r="N96" t="s">
         <v>30</v>
       </c>
-      <c r="P96" s="33" t="s">
+      <c r="P96" t="s">
         <v>30</v>
       </c>
-      <c r="R96" s="31">
+      <c r="R96">
         <v>35</v>
       </c>
-      <c r="T96" s="31">
+      <c r="T96">
         <v>35</v>
       </c>
     </row>
@@ -14764,8 +14770,8 @@
       </c>
       <c r="F99" s="13"/>
       <c r="G99" s="12">
-        <f>SUM(H98:H99)</f>
-        <v>100</v>
+        <f>SUM(H98)</f>
+        <v>95</v>
       </c>
       <c r="H99" s="12">
         <v>5</v>
@@ -14848,52 +14854,52 @@
         <v>0.58611111111111114</v>
       </c>
     </row>
-    <row r="101" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A101" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B101" s="31" t="s">
+      <c r="B101" t="s">
         <v>73</v>
       </c>
-      <c r="C101" s="31" t="s">
+      <c r="C101" t="s">
         <v>52</v>
       </c>
-      <c r="D101" s="31">
+      <c r="D101">
         <v>1</v>
       </c>
-      <c r="E101" s="31">
+      <c r="E101">
         <v>12</v>
       </c>
-      <c r="F101" s="32"/>
-      <c r="H101" s="31">
+      <c r="F101" s="9"/>
+      <c r="H101">
         <v>20</v>
       </c>
-      <c r="I101" s="31" t="s">
+      <c r="I101" t="s">
         <v>26</v>
       </c>
-      <c r="J101" s="31">
+      <c r="J101">
         <f t="shared" si="1"/>
         <v>77.25</v>
       </c>
-      <c r="K101" s="31" t="s">
+      <c r="K101" t="s">
         <v>26</v>
       </c>
-      <c r="L101" s="31">
+      <c r="L101">
         <v>64</v>
       </c>
-      <c r="N101" s="31">
+      <c r="N101">
         <v>95</v>
       </c>
-      <c r="P101" s="31">
+      <c r="P101">
         <v>72</v>
       </c>
-      <c r="R101" s="31">
+      <c r="R101">
         <v>78</v>
       </c>
-      <c r="T101" s="31">
+      <c r="T101">
         <v>56.5</v>
       </c>
-      <c r="W101" s="31" t="s">
+      <c r="W101" t="s">
         <v>111</v>
       </c>
     </row>
@@ -14915,8 +14921,8 @@
       </c>
       <c r="F102" s="13"/>
       <c r="G102" s="12">
-        <f>SUM(H100:H102)</f>
-        <v>110</v>
+        <f>SUM(H100:H101)</f>
+        <v>80</v>
       </c>
       <c r="H102" s="12">
         <v>30</v>
@@ -14996,83 +15002,83 @@
         <v>0.5756944444444444</v>
       </c>
     </row>
-    <row r="104" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A104" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B104" s="31" t="s">
+      <c r="B104" t="s">
         <v>73</v>
       </c>
-      <c r="C104" s="31" t="s">
+      <c r="C104" t="s">
         <v>52</v>
       </c>
-      <c r="D104" s="31">
+      <c r="D104">
         <v>1</v>
       </c>
-      <c r="E104" s="31">
+      <c r="E104">
         <v>18</v>
       </c>
-      <c r="F104" s="32"/>
-      <c r="H104" s="31">
+      <c r="F104" s="9"/>
+      <c r="H104">
         <v>10</v>
       </c>
-      <c r="I104" s="31" t="s">
+      <c r="I104" t="s">
         <v>31</v>
       </c>
-      <c r="J104" s="31" t="e">
+      <c r="J104" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T104" s="31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="T104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A105" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B105" s="31" t="s">
+      <c r="B105" t="s">
         <v>73</v>
       </c>
-      <c r="C105" s="31" t="s">
+      <c r="C105" t="s">
         <v>52</v>
       </c>
-      <c r="D105" s="31">
+      <c r="D105">
         <v>1</v>
       </c>
-      <c r="E105" s="31">
+      <c r="E105">
         <v>18</v>
       </c>
-      <c r="F105" s="32"/>
-      <c r="H105" s="31">
+      <c r="F105" s="9"/>
+      <c r="H105">
         <v>45</v>
       </c>
-      <c r="I105" s="31" t="s">
+      <c r="I105" t="s">
         <v>26</v>
       </c>
-      <c r="J105" s="31">
+      <c r="J105">
         <f t="shared" si="1"/>
         <v>68.25</v>
       </c>
-      <c r="K105" s="31" t="s">
+      <c r="K105" t="s">
         <v>26</v>
       </c>
-      <c r="L105" s="31">
+      <c r="L105">
         <v>71</v>
       </c>
-      <c r="N105" s="31">
+      <c r="N105">
         <v>68</v>
       </c>
-      <c r="P105" s="31">
+      <c r="P105">
         <v>66</v>
       </c>
-      <c r="R105" s="31">
+      <c r="R105">
         <v>68</v>
       </c>
-      <c r="T105" s="31">
+      <c r="T105">
         <v>71</v>
       </c>
-      <c r="V105" s="31" t="s">
+      <c r="V105" t="s">
         <v>112</v>
       </c>
     </row>
@@ -15094,8 +15100,8 @@
       </c>
       <c r="F106" s="13"/>
       <c r="G106" s="12">
-        <f>SUM(H103:H106)</f>
-        <v>125</v>
+        <f>SUM(H103:H105)</f>
+        <v>90</v>
       </c>
       <c r="H106" s="12">
         <v>35</v>
@@ -15178,98 +15184,98 @@
         <v>0.5625</v>
       </c>
     </row>
-    <row r="108" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A108" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B108" s="31" t="s">
+      <c r="B108" t="s">
         <v>73</v>
       </c>
-      <c r="C108" s="31" t="s">
+      <c r="C108" t="s">
         <v>52</v>
       </c>
-      <c r="D108" s="31">
+      <c r="D108">
         <v>1</v>
       </c>
-      <c r="E108" s="31">
-        <v>24</v>
-      </c>
-      <c r="F108" s="32"/>
-      <c r="H108" s="31">
+      <c r="E108">
+        <v>24</v>
+      </c>
+      <c r="F108" s="9"/>
+      <c r="H108">
         <v>80</v>
       </c>
-      <c r="I108" s="31" t="s">
+      <c r="I108" t="s">
         <v>36</v>
       </c>
-      <c r="J108" s="31">
+      <c r="J108">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="K108" s="33" t="s">
+      <c r="K108" t="s">
         <v>36</v>
       </c>
-      <c r="L108" s="33">
+      <c r="L108">
         <v>27</v>
       </c>
-      <c r="N108" s="33">
-        <v>23</v>
-      </c>
-      <c r="P108" s="33">
+      <c r="N108">
+        <v>23</v>
+      </c>
+      <c r="P108">
         <v>20</v>
       </c>
-      <c r="R108" s="33">
+      <c r="R108">
         <v>30</v>
       </c>
-      <c r="T108" s="31">
+      <c r="T108">
         <v>30</v>
       </c>
-      <c r="V108" s="31" t="s">
+      <c r="V108" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A109" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B109" s="31" t="s">
+      <c r="B109" t="s">
         <v>73</v>
       </c>
-      <c r="C109" s="31" t="s">
+      <c r="C109" t="s">
         <v>52</v>
       </c>
-      <c r="D109" s="31">
+      <c r="D109">
         <v>1</v>
       </c>
-      <c r="E109" s="31">
-        <v>24</v>
-      </c>
-      <c r="F109" s="32"/>
-      <c r="H109" s="31">
+      <c r="E109">
+        <v>24</v>
+      </c>
+      <c r="F109" s="9"/>
+      <c r="H109">
         <v>20</v>
       </c>
-      <c r="I109" s="31" t="s">
+      <c r="I109" t="s">
         <v>26</v>
       </c>
-      <c r="J109" s="31">
+      <c r="J109">
         <f t="shared" si="1"/>
         <v>64.25</v>
       </c>
-      <c r="K109" s="31" t="s">
+      <c r="K109" t="s">
         <v>26</v>
       </c>
-      <c r="L109" s="31">
+      <c r="L109">
         <v>71.5</v>
       </c>
-      <c r="N109" s="31">
+      <c r="N109">
         <v>63.5</v>
       </c>
-      <c r="P109" s="31">
+      <c r="P109">
         <v>55</v>
       </c>
-      <c r="R109" s="31">
+      <c r="R109">
         <v>67</v>
       </c>
-      <c r="T109" s="31">
+      <c r="T109">
         <v>71.5</v>
       </c>
     </row>
@@ -15339,52 +15345,52 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A112" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B112" s="31" t="s">
+      <c r="B112" t="s">
         <v>73</v>
       </c>
-      <c r="C112" s="31" t="s">
+      <c r="C112" t="s">
         <v>52</v>
       </c>
-      <c r="D112" s="31">
+      <c r="D112">
         <v>1</v>
       </c>
-      <c r="E112" s="31">
+      <c r="E112">
         <v>48</v>
       </c>
-      <c r="F112" s="32"/>
-      <c r="H112" s="31">
+      <c r="F112" s="9"/>
+      <c r="H112">
         <v>90</v>
       </c>
-      <c r="I112" s="31" t="s">
+      <c r="I112" t="s">
         <v>31</v>
       </c>
-      <c r="J112" s="31">
+      <c r="J112">
         <f t="shared" si="1"/>
         <v>30.125</v>
       </c>
-      <c r="K112" s="31" t="s">
+      <c r="K112" t="s">
         <v>31</v>
       </c>
-      <c r="L112" s="31">
+      <c r="L112">
         <v>30</v>
       </c>
-      <c r="N112" s="31">
+      <c r="N112">
         <v>33.5</v>
       </c>
-      <c r="P112" s="31">
+      <c r="P112">
         <v>30</v>
       </c>
-      <c r="R112" s="31">
+      <c r="R112">
         <v>27</v>
       </c>
-      <c r="T112" s="31">
+      <c r="T112">
         <v>33.5</v>
       </c>
-      <c r="V112" s="34">
+      <c r="V112" s="16">
         <v>0.55277777777777781</v>
       </c>
     </row>
@@ -15406,8 +15412,8 @@
       </c>
       <c r="F113" s="13"/>
       <c r="G113" s="12">
-        <f>SUM(H111:H113)</f>
-        <v>100</v>
+        <f>SUM(H112:H113)</f>
+        <v>95</v>
       </c>
       <c r="H113" s="12">
         <v>5</v>
@@ -15502,80 +15508,80 @@
         <v>0.62708333333333333</v>
       </c>
     </row>
-    <row r="115" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A115" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B115" s="31" t="s">
+      <c r="B115" t="s">
         <v>73</v>
       </c>
-      <c r="C115" s="31" t="s">
+      <c r="C115" t="s">
         <v>52</v>
       </c>
-      <c r="D115" s="31">
-        <v>2</v>
-      </c>
-      <c r="E115" s="31">
+      <c r="D115">
+        <v>2</v>
+      </c>
+      <c r="E115">
         <v>0.5</v>
       </c>
-      <c r="F115" s="32"/>
-      <c r="H115" s="31">
+      <c r="F115" s="9"/>
+      <c r="H115">
         <v>75</v>
       </c>
-      <c r="I115" s="31" t="s">
+      <c r="I115" t="s">
         <v>36</v>
       </c>
-      <c r="J115" s="31">
+      <c r="J115">
         <f t="shared" si="1"/>
         <v>16.25</v>
       </c>
-      <c r="L115" s="33">
+      <c r="L115">
         <v>19</v>
       </c>
-      <c r="N115" s="33">
+      <c r="N115">
         <v>12</v>
       </c>
-      <c r="P115" s="31">
+      <c r="P115">
         <v>18</v>
       </c>
-      <c r="R115" s="31">
+      <c r="R115">
         <v>16</v>
       </c>
-      <c r="T115" s="31">
+      <c r="T115">
         <v>19</v>
       </c>
-      <c r="W115" s="31" t="s">
+      <c r="W115" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="116" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A116" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B116" s="31" t="s">
+      <c r="B116" t="s">
         <v>73</v>
       </c>
-      <c r="C116" s="31" t="s">
+      <c r="C116" t="s">
         <v>52</v>
       </c>
-      <c r="D116" s="31">
-        <v>2</v>
-      </c>
-      <c r="E116" s="31">
+      <c r="D116">
+        <v>2</v>
+      </c>
+      <c r="E116">
         <v>0.5</v>
       </c>
-      <c r="F116" s="32"/>
-      <c r="H116" s="31">
+      <c r="F116" s="9"/>
+      <c r="H116">
         <v>15</v>
       </c>
-      <c r="I116" s="31" t="s">
+      <c r="I116" t="s">
         <v>31</v>
       </c>
-      <c r="J116" s="31" t="e">
+      <c r="J116" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T116" s="31">
+      <c r="T116">
         <v>0</v>
       </c>
     </row>
@@ -15597,8 +15603,8 @@
       </c>
       <c r="F117" s="13"/>
       <c r="G117" s="12">
-        <f>SUM(H114:H117)</f>
-        <v>115</v>
+        <f>SUM(H114:H116)</f>
+        <v>110</v>
       </c>
       <c r="H117" s="12">
         <v>5</v>
@@ -15678,95 +15684,95 @@
         <v>0.63541666666666663</v>
       </c>
     </row>
-    <row r="119" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A119" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B119" s="31" t="s">
+      <c r="B119" t="s">
         <v>73</v>
       </c>
-      <c r="C119" s="31" t="s">
+      <c r="C119" t="s">
         <v>52</v>
       </c>
-      <c r="D119" s="31">
-        <v>2</v>
-      </c>
-      <c r="E119" s="31">
-        <v>2</v>
-      </c>
-      <c r="F119" s="32"/>
-      <c r="H119" s="31">
+      <c r="D119">
+        <v>2</v>
+      </c>
+      <c r="E119">
+        <v>2</v>
+      </c>
+      <c r="F119" s="9"/>
+      <c r="H119">
         <v>75</v>
       </c>
-      <c r="I119" s="31" t="s">
+      <c r="I119" t="s">
         <v>36</v>
       </c>
-      <c r="J119" s="31">
+      <c r="J119">
         <f t="shared" ref="J119:J179" si="2">AVERAGE(L119, N119, P119, R119)</f>
         <v>16.375</v>
       </c>
-      <c r="K119" s="31" t="s">
+      <c r="K119" t="s">
         <v>36</v>
       </c>
-      <c r="L119" s="31">
+      <c r="L119">
         <v>19</v>
       </c>
-      <c r="N119" s="31">
+      <c r="N119">
         <v>15.5</v>
       </c>
-      <c r="P119" s="31">
+      <c r="P119">
         <v>14</v>
       </c>
-      <c r="R119" s="31">
+      <c r="R119">
         <v>17</v>
       </c>
-      <c r="T119" s="31">
+      <c r="T119">
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A120" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B120" s="31" t="s">
+      <c r="B120" t="s">
         <v>73</v>
       </c>
-      <c r="C120" s="31" t="s">
+      <c r="C120" t="s">
         <v>52</v>
       </c>
-      <c r="D120" s="31">
-        <v>2</v>
-      </c>
-      <c r="E120" s="31">
-        <v>2</v>
-      </c>
-      <c r="F120" s="32"/>
-      <c r="H120" s="31">
+      <c r="D120">
+        <v>2</v>
+      </c>
+      <c r="E120">
+        <v>2</v>
+      </c>
+      <c r="F120" s="9"/>
+      <c r="H120">
         <v>65</v>
       </c>
-      <c r="I120" s="31" t="s">
+      <c r="I120" t="s">
         <v>31</v>
       </c>
-      <c r="J120" s="31">
+      <c r="J120">
         <f t="shared" si="2"/>
         <v>21.333333333333332</v>
       </c>
-      <c r="K120" s="31" t="s">
+      <c r="K120" t="s">
         <v>31</v>
       </c>
-      <c r="L120" s="31" t="s">
+      <c r="L120" t="s">
         <v>30</v>
       </c>
-      <c r="N120" s="31">
+      <c r="N120">
         <v>20</v>
       </c>
-      <c r="P120" s="31">
-        <v>28</v>
-      </c>
-      <c r="R120" s="31">
+      <c r="P120">
+        <v>28</v>
+      </c>
+      <c r="R120">
         <v>16</v>
       </c>
-      <c r="T120" s="31">
+      <c r="T120">
         <v>28</v>
       </c>
     </row>
@@ -15788,8 +15794,8 @@
       </c>
       <c r="F121" s="13"/>
       <c r="G121" s="12">
-        <f>SUM(H118:H121)</f>
-        <v>165</v>
+        <f>SUM(H118:H120)</f>
+        <v>160</v>
       </c>
       <c r="H121" s="12">
         <v>5</v>
@@ -15869,126 +15875,126 @@
         <v>0.6430555555555556</v>
       </c>
     </row>
-    <row r="123" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A123" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B123" s="31" t="s">
+      <c r="B123" t="s">
         <v>73</v>
       </c>
-      <c r="C123" s="31" t="s">
+      <c r="C123" t="s">
         <v>52</v>
       </c>
-      <c r="D123" s="31">
-        <v>2</v>
-      </c>
-      <c r="E123" s="31">
+      <c r="D123">
+        <v>2</v>
+      </c>
+      <c r="E123">
         <v>6</v>
       </c>
-      <c r="F123" s="32"/>
-      <c r="H123" s="31">
+      <c r="F123" s="9"/>
+      <c r="H123">
         <v>50</v>
       </c>
-      <c r="I123" s="31" t="s">
+      <c r="I123" t="s">
         <v>36</v>
       </c>
-      <c r="J123" s="31">
+      <c r="J123">
         <f t="shared" si="2"/>
         <v>21.875</v>
       </c>
-      <c r="L123" s="33">
+      <c r="L123">
         <v>20</v>
       </c>
-      <c r="N123" s="33">
+      <c r="N123">
         <v>18</v>
       </c>
-      <c r="P123" s="33">
+      <c r="P123">
         <v>25</v>
       </c>
-      <c r="R123" s="33">
+      <c r="R123">
         <v>24.5</v>
       </c>
-      <c r="T123" s="31">
+      <c r="T123">
         <v>25</v>
       </c>
-      <c r="W123" s="31" t="s">
+      <c r="W123" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="124" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A124" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B124" s="31" t="s">
+      <c r="B124" t="s">
         <v>73</v>
       </c>
-      <c r="C124" s="31" t="s">
+      <c r="C124" t="s">
         <v>52</v>
       </c>
-      <c r="D124" s="31">
-        <v>2</v>
-      </c>
-      <c r="E124" s="31">
+      <c r="D124">
+        <v>2</v>
+      </c>
+      <c r="E124">
         <v>6</v>
       </c>
-      <c r="F124" s="32"/>
-      <c r="H124" s="31">
+      <c r="F124" s="9"/>
+      <c r="H124">
         <v>30</v>
       </c>
-      <c r="I124" s="31" t="s">
+      <c r="I124" t="s">
         <v>31</v>
       </c>
-      <c r="J124" s="31" t="e">
+      <c r="J124" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T124" s="31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="T124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A125" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B125" s="31" t="s">
+      <c r="B125" t="s">
         <v>73</v>
       </c>
-      <c r="C125" s="31" t="s">
+      <c r="C125" t="s">
         <v>52</v>
       </c>
-      <c r="D125" s="31">
-        <v>2</v>
-      </c>
-      <c r="E125" s="31">
+      <c r="D125">
+        <v>2</v>
+      </c>
+      <c r="E125">
         <v>6</v>
       </c>
-      <c r="F125" s="32"/>
-      <c r="H125" s="31">
+      <c r="F125" s="9"/>
+      <c r="H125">
         <v>10</v>
       </c>
-      <c r="I125" s="31" t="s">
+      <c r="I125" t="s">
         <v>26</v>
       </c>
-      <c r="J125" s="31">
+      <c r="J125">
         <f t="shared" si="2"/>
         <v>53.166666666666664</v>
       </c>
-      <c r="K125" s="31" t="s">
+      <c r="K125" t="s">
         <v>26</v>
       </c>
-      <c r="L125" s="31">
+      <c r="L125">
         <v>59.5</v>
       </c>
-      <c r="N125" s="31">
+      <c r="N125">
         <v>40</v>
       </c>
-      <c r="P125" s="31" t="s">
+      <c r="P125" t="s">
         <v>30</v>
       </c>
-      <c r="R125" s="31">
+      <c r="R125">
         <v>60</v>
       </c>
-      <c r="T125" s="31">
+      <c r="T125">
         <v>60</v>
       </c>
     </row>
@@ -16010,8 +16016,8 @@
       </c>
       <c r="F126" s="13"/>
       <c r="G126" s="12">
-        <f>SUM(H122:H126)</f>
-        <v>135</v>
+        <f>SUM(H122:H125)</f>
+        <v>130</v>
       </c>
       <c r="H126" s="12">
         <v>5</v>
@@ -16061,144 +16067,144 @@
         <v>0.65208333333333335</v>
       </c>
     </row>
-    <row r="128" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A128" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B128" s="31" t="s">
+      <c r="B128" t="s">
         <v>73</v>
       </c>
-      <c r="C128" s="31" t="s">
+      <c r="C128" t="s">
         <v>52</v>
       </c>
-      <c r="D128" s="31">
-        <v>2</v>
-      </c>
-      <c r="E128" s="31">
+      <c r="D128">
+        <v>2</v>
+      </c>
+      <c r="E128">
         <v>12</v>
       </c>
-      <c r="F128" s="32"/>
-      <c r="H128" s="31">
+      <c r="F128" s="9"/>
+      <c r="H128">
         <v>35</v>
       </c>
-      <c r="I128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J128" s="31">
+      <c r="I128" t="s">
+        <v>28</v>
+      </c>
+      <c r="J128">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="K128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L128" s="31">
+      <c r="K128" t="s">
+        <v>28</v>
+      </c>
+      <c r="L128">
         <v>64</v>
       </c>
-      <c r="M128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N128" s="31">
+      <c r="M128" t="s">
+        <v>28</v>
+      </c>
+      <c r="N128">
         <v>36</v>
       </c>
-      <c r="O128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P128" s="31">
+      <c r="O128" t="s">
+        <v>28</v>
+      </c>
+      <c r="P128">
         <v>40</v>
       </c>
-      <c r="Q128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R128" s="31">
+      <c r="Q128" t="s">
+        <v>28</v>
+      </c>
+      <c r="R128">
         <v>52</v>
       </c>
-      <c r="S128" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T128" s="31">
+      <c r="S128" t="s">
+        <v>28</v>
+      </c>
+      <c r="T128">
         <v>64</v>
       </c>
-      <c r="U128" s="31" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="129" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="U128" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A129" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B129" s="31" t="s">
+      <c r="B129" t="s">
         <v>73</v>
       </c>
-      <c r="C129" s="31" t="s">
+      <c r="C129" t="s">
         <v>52</v>
       </c>
-      <c r="D129" s="31">
-        <v>2</v>
-      </c>
-      <c r="E129" s="31">
+      <c r="D129">
+        <v>2</v>
+      </c>
+      <c r="E129">
         <v>12</v>
       </c>
-      <c r="F129" s="32"/>
-      <c r="H129" s="31">
+      <c r="F129" s="9"/>
+      <c r="H129">
         <v>55</v>
       </c>
-      <c r="I129" s="31" t="s">
+      <c r="I129" t="s">
         <v>36</v>
       </c>
-      <c r="J129" s="31">
+      <c r="J129">
         <f t="shared" si="2"/>
         <v>20.75</v>
       </c>
-      <c r="L129" s="31">
+      <c r="L129">
         <v>18</v>
       </c>
-      <c r="N129" s="31">
+      <c r="N129">
         <v>20</v>
       </c>
-      <c r="P129" s="31">
+      <c r="P129">
         <v>22</v>
       </c>
-      <c r="R129" s="31">
-        <v>23</v>
-      </c>
-      <c r="T129" s="31">
-        <v>23</v>
-      </c>
-      <c r="W129" s="31" t="s">
+      <c r="R129">
+        <v>23</v>
+      </c>
+      <c r="T129">
+        <v>23</v>
+      </c>
+      <c r="W129" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="130" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A130" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B130" s="31" t="s">
+      <c r="B130" t="s">
         <v>73</v>
       </c>
-      <c r="C130" s="31" t="s">
+      <c r="C130" t="s">
         <v>52</v>
       </c>
-      <c r="D130" s="31">
-        <v>2</v>
-      </c>
-      <c r="E130" s="31">
+      <c r="D130">
+        <v>2</v>
+      </c>
+      <c r="E130">
         <v>12</v>
       </c>
-      <c r="F130" s="32"/>
-      <c r="H130" s="31">
+      <c r="F130" s="9"/>
+      <c r="H130">
         <v>10</v>
       </c>
-      <c r="I130" s="31" t="s">
+      <c r="I130" t="s">
         <v>31</v>
       </c>
-      <c r="J130" s="31" t="e">
+      <c r="J130" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T130" s="31">
-        <v>0</v>
-      </c>
-      <c r="W130" s="31" t="s">
+      <c r="T130">
+        <v>0</v>
+      </c>
+      <c r="W130" t="s">
         <v>118</v>
       </c>
     </row>
@@ -16220,8 +16226,8 @@
       </c>
       <c r="F131" s="13"/>
       <c r="G131" s="12">
-        <f>SUM(H127:H131)</f>
-        <v>125</v>
+        <f>SUM(H128:H131)</f>
+        <v>115</v>
       </c>
       <c r="H131" s="12">
         <v>15</v>
@@ -16286,110 +16292,110 @@
         <v>0.66388888888888886</v>
       </c>
     </row>
-    <row r="133" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A133" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B133" s="31" t="s">
+      <c r="B133" t="s">
         <v>73</v>
       </c>
-      <c r="C133" s="31" t="s">
+      <c r="C133" t="s">
         <v>52</v>
       </c>
-      <c r="D133" s="31">
-        <v>2</v>
-      </c>
-      <c r="E133" s="31">
+      <c r="D133">
+        <v>2</v>
+      </c>
+      <c r="E133">
         <v>18</v>
       </c>
-      <c r="F133" s="32"/>
-      <c r="H133" s="31">
+      <c r="F133" s="9"/>
+      <c r="H133">
         <v>25</v>
       </c>
-      <c r="I133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J133" s="31">
+      <c r="I133" t="s">
+        <v>28</v>
+      </c>
+      <c r="J133">
         <f t="shared" si="2"/>
         <v>48.75</v>
       </c>
-      <c r="K133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L133" s="31">
+      <c r="K133" t="s">
+        <v>28</v>
+      </c>
+      <c r="L133">
         <v>45</v>
       </c>
-      <c r="M133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N133" s="31">
+      <c r="M133" t="s">
+        <v>28</v>
+      </c>
+      <c r="N133">
         <v>51</v>
       </c>
-      <c r="O133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P133" s="31">
+      <c r="O133" t="s">
+        <v>28</v>
+      </c>
+      <c r="P133">
         <v>50</v>
       </c>
-      <c r="Q133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R133" s="31">
+      <c r="Q133" t="s">
+        <v>28</v>
+      </c>
+      <c r="R133">
         <v>49</v>
       </c>
-      <c r="S133" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T133" s="31">
+      <c r="S133" t="s">
+        <v>28</v>
+      </c>
+      <c r="T133">
         <v>51</v>
       </c>
-      <c r="U133" s="31" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="134" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="U133" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A134" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B134" s="31" t="s">
+      <c r="B134" t="s">
         <v>73</v>
       </c>
-      <c r="C134" s="31" t="s">
+      <c r="C134" t="s">
         <v>52</v>
       </c>
-      <c r="D134" s="31">
-        <v>2</v>
-      </c>
-      <c r="E134" s="31">
+      <c r="D134">
+        <v>2</v>
+      </c>
+      <c r="E134">
         <v>18</v>
       </c>
-      <c r="F134" s="32"/>
-      <c r="H134" s="31">
+      <c r="F134" s="9"/>
+      <c r="H134">
         <v>35</v>
       </c>
-      <c r="I134" s="31" t="s">
+      <c r="I134" t="s">
         <v>26</v>
       </c>
-      <c r="J134" s="31">
+      <c r="J134">
         <f t="shared" si="2"/>
         <v>55.25</v>
       </c>
-      <c r="K134" s="31" t="s">
+      <c r="K134" t="s">
         <v>26</v>
       </c>
-      <c r="L134" s="31">
+      <c r="L134">
         <v>57</v>
       </c>
-      <c r="N134" s="31">
+      <c r="N134">
         <v>52</v>
       </c>
-      <c r="P134" s="31">
+      <c r="P134">
         <v>50</v>
       </c>
-      <c r="R134" s="31">
+      <c r="R134">
         <v>62</v>
       </c>
-      <c r="T134" s="31">
+      <c r="T134">
         <v>62</v>
       </c>
     </row>
@@ -16411,8 +16417,8 @@
       </c>
       <c r="F135" s="13"/>
       <c r="G135" s="12">
-        <f>SUM(H132:H135)</f>
-        <v>120</v>
+        <f>SUM(H133:H135)</f>
+        <v>105</v>
       </c>
       <c r="H135" s="12">
         <v>45</v>
@@ -16471,147 +16477,147 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A137" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B137" s="31" t="s">
+      <c r="B137" t="s">
         <v>73</v>
       </c>
-      <c r="C137" s="31" t="s">
+      <c r="C137" t="s">
         <v>52</v>
       </c>
-      <c r="D137" s="31">
-        <v>2</v>
-      </c>
-      <c r="E137" s="31">
-        <v>24</v>
-      </c>
-      <c r="F137" s="32"/>
-      <c r="H137" s="31">
+      <c r="D137">
+        <v>2</v>
+      </c>
+      <c r="E137">
+        <v>24</v>
+      </c>
+      <c r="F137" s="9"/>
+      <c r="H137">
         <v>20</v>
       </c>
-      <c r="I137" s="31" t="s">
+      <c r="I137" t="s">
         <v>26</v>
       </c>
-      <c r="J137" s="31">
+      <c r="J137">
         <f t="shared" si="2"/>
         <v>53.75</v>
       </c>
-      <c r="K137" s="31" t="s">
+      <c r="K137" t="s">
         <v>26</v>
       </c>
-      <c r="L137" s="31">
+      <c r="L137">
         <v>57</v>
       </c>
-      <c r="N137" s="31">
+      <c r="N137">
         <v>55</v>
       </c>
-      <c r="P137" s="31">
+      <c r="P137">
         <v>51</v>
       </c>
-      <c r="R137" s="31">
+      <c r="R137">
         <v>52</v>
       </c>
-      <c r="T137" s="31">
+      <c r="T137">
         <v>57</v>
       </c>
-      <c r="W137" s="31" t="s">
+      <c r="W137" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="138" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A138" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B138" s="31" t="s">
+      <c r="B138" t="s">
         <v>73</v>
       </c>
-      <c r="C138" s="31" t="s">
+      <c r="C138" t="s">
         <v>52</v>
       </c>
-      <c r="D138" s="31">
-        <v>2</v>
-      </c>
-      <c r="E138" s="31">
-        <v>24</v>
-      </c>
-      <c r="F138" s="32"/>
-      <c r="H138" s="31">
+      <c r="D138">
+        <v>2</v>
+      </c>
+      <c r="E138">
+        <v>24</v>
+      </c>
+      <c r="F138" s="9"/>
+      <c r="H138">
         <v>25</v>
       </c>
-      <c r="I138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J138" s="31">
+      <c r="I138" t="s">
+        <v>28</v>
+      </c>
+      <c r="J138">
         <f t="shared" si="2"/>
         <v>33.75</v>
       </c>
-      <c r="K138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L138" s="31">
+      <c r="K138" t="s">
+        <v>28</v>
+      </c>
+      <c r="L138">
         <v>33</v>
       </c>
-      <c r="M138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N138" s="31">
+      <c r="M138" t="s">
+        <v>28</v>
+      </c>
+      <c r="N138">
         <v>29</v>
       </c>
-      <c r="O138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P138" s="31">
+      <c r="O138" t="s">
+        <v>28</v>
+      </c>
+      <c r="P138">
         <v>38</v>
       </c>
-      <c r="Q138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R138" s="31">
+      <c r="Q138" t="s">
+        <v>28</v>
+      </c>
+      <c r="R138">
         <v>35</v>
       </c>
-      <c r="S138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T138" s="31">
+      <c r="S138" t="s">
+        <v>28</v>
+      </c>
+      <c r="T138">
         <v>38</v>
       </c>
-      <c r="U138" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="V138" s="34">
+      <c r="U138" t="s">
+        <v>28</v>
+      </c>
+      <c r="V138" s="16">
         <v>0.6743055555555556</v>
       </c>
     </row>
-    <row r="139" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A139" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B139" s="31" t="s">
+      <c r="B139" t="s">
         <v>73</v>
       </c>
-      <c r="C139" s="31" t="s">
+      <c r="C139" t="s">
         <v>52</v>
       </c>
-      <c r="D139" s="31">
-        <v>2</v>
-      </c>
-      <c r="E139" s="31">
-        <v>24</v>
-      </c>
-      <c r="F139" s="32"/>
-      <c r="H139" s="31">
+      <c r="D139">
+        <v>2</v>
+      </c>
+      <c r="E139">
+        <v>24</v>
+      </c>
+      <c r="F139" s="9"/>
+      <c r="H139">
         <v>10</v>
       </c>
-      <c r="I139" s="31" t="s">
+      <c r="I139" t="s">
         <v>31</v>
       </c>
-      <c r="J139" s="31" t="e">
+      <c r="J139" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T139" s="31">
+      <c r="T139">
         <v>0</v>
       </c>
     </row>
@@ -16633,8 +16639,8 @@
       </c>
       <c r="F140" s="13"/>
       <c r="G140" s="12">
-        <f>SUM(H136:H140)</f>
-        <v>125</v>
+        <f>SUM(H137:H140)</f>
+        <v>120</v>
       </c>
       <c r="H140" s="12">
         <v>65</v>
@@ -16699,83 +16705,83 @@
         <v>0.68541666666666667</v>
       </c>
     </row>
-    <row r="142" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A142" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B142" s="31" t="s">
+      <c r="B142" t="s">
         <v>73</v>
       </c>
-      <c r="C142" s="31" t="s">
+      <c r="C142" t="s">
         <v>52</v>
       </c>
-      <c r="D142" s="31">
-        <v>2</v>
-      </c>
-      <c r="E142" s="31">
+      <c r="D142">
+        <v>2</v>
+      </c>
+      <c r="E142">
         <v>48</v>
       </c>
-      <c r="F142" s="32"/>
-      <c r="H142" s="31">
+      <c r="F142" s="9"/>
+      <c r="H142">
         <v>35</v>
       </c>
-      <c r="I142" s="31" t="s">
+      <c r="I142" t="s">
         <v>36</v>
       </c>
-      <c r="J142" s="31" t="e">
+      <c r="J142" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="T142" s="31">
-        <v>0</v>
-      </c>
-      <c r="W142" s="31" t="s">
+      <c r="T142">
+        <v>0</v>
+      </c>
+      <c r="W142" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="143" spans="1:23" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A143" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B143" s="31" t="s">
+      <c r="B143" t="s">
         <v>73</v>
       </c>
-      <c r="C143" s="31" t="s">
+      <c r="C143" t="s">
         <v>52</v>
       </c>
-      <c r="D143" s="31">
-        <v>2</v>
-      </c>
-      <c r="E143" s="31">
+      <c r="D143">
+        <v>2</v>
+      </c>
+      <c r="E143">
         <v>48</v>
       </c>
-      <c r="F143" s="32"/>
-      <c r="H143" s="31">
+      <c r="F143" s="9"/>
+      <c r="H143">
         <v>90</v>
       </c>
-      <c r="I143" s="31" t="s">
+      <c r="I143" t="s">
         <v>31</v>
       </c>
-      <c r="J143" s="31">
+      <c r="J143">
         <f t="shared" si="2"/>
         <v>31</v>
       </c>
-      <c r="K143" s="31" t="s">
+      <c r="K143" t="s">
         <v>31</v>
       </c>
-      <c r="L143" s="31">
+      <c r="L143">
         <v>27</v>
       </c>
-      <c r="N143" s="31">
+      <c r="N143">
         <v>33</v>
       </c>
-      <c r="P143" s="31">
+      <c r="P143">
         <v>31</v>
       </c>
-      <c r="R143" s="31">
+      <c r="R143">
         <v>33</v>
       </c>
-      <c r="T143" s="31">
+      <c r="T143">
         <v>33</v>
       </c>
     </row>
@@ -16797,8 +16803,8 @@
       </c>
       <c r="F144" s="13"/>
       <c r="G144" s="12">
-        <f>SUM(H141:H144)</f>
-        <v>135</v>
+        <f>SUM(H142:H144)</f>
+        <v>130</v>
       </c>
       <c r="H144" s="12">
         <v>5</v>
@@ -16893,46 +16899,46 @@
         <v>0.43541666666666667</v>
       </c>
     </row>
-    <row r="146" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A146" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B146" s="31" t="s">
+      <c r="B146" t="s">
         <v>73</v>
       </c>
-      <c r="C146" s="31" t="s">
+      <c r="C146" t="s">
         <v>60</v>
       </c>
-      <c r="D146" s="31">
+      <c r="D146">
         <v>1</v>
       </c>
-      <c r="E146" s="31">
+      <c r="E146">
         <v>0.5</v>
       </c>
-      <c r="F146" s="32"/>
-      <c r="H146" s="31">
+      <c r="F146" s="9"/>
+      <c r="H146">
         <v>35</v>
       </c>
-      <c r="I146" s="31" t="s">
+      <c r="I146" t="s">
         <v>26</v>
       </c>
-      <c r="J146" s="31">
+      <c r="J146">
         <f t="shared" si="2"/>
         <v>67.125</v>
       </c>
-      <c r="L146" s="33">
+      <c r="L146">
         <v>76</v>
       </c>
-      <c r="N146" s="31">
+      <c r="N146">
         <v>69.5</v>
       </c>
-      <c r="P146" s="31">
+      <c r="P146">
         <v>70</v>
       </c>
-      <c r="R146" s="31">
+      <c r="R146">
         <v>53</v>
       </c>
-      <c r="T146" s="31">
+      <c r="T146">
         <v>76</v>
       </c>
     </row>
@@ -16954,8 +16960,8 @@
       </c>
       <c r="F147" s="13"/>
       <c r="G147" s="12">
-        <f>SUM(H145:H147)</f>
-        <v>110</v>
+        <f>SUM(H145:H146)</f>
+        <v>70</v>
       </c>
       <c r="H147" s="12">
         <v>40</v>
@@ -17053,8 +17059,8 @@
       </c>
       <c r="F149" s="13"/>
       <c r="G149" s="12">
-        <f>SUM(H148:H149)</f>
-        <v>100</v>
+        <f>SUM(H148)</f>
+        <v>75</v>
       </c>
       <c r="H149" s="12">
         <v>25</v>
@@ -17119,8 +17125,8 @@
       </c>
       <c r="F151" s="13"/>
       <c r="G151" s="12">
-        <f>SUM(H150:H151)</f>
-        <v>100</v>
+        <f>SUM(H151)</f>
+        <v>60</v>
       </c>
       <c r="H151" s="12">
         <v>60</v>
@@ -17251,8 +17257,8 @@
       </c>
       <c r="F153" s="13"/>
       <c r="G153" s="12">
-        <f>SUM(H152:H153)</f>
-        <v>100</v>
+        <f>SUM(H152)</f>
+        <v>65</v>
       </c>
       <c r="H153" s="12">
         <v>35</v>
@@ -17350,8 +17356,8 @@
       </c>
       <c r="F155" s="13"/>
       <c r="G155" s="12">
-        <f>SUM(H154:H155)</f>
-        <v>100</v>
+        <f>SUM(H154)</f>
+        <v>80</v>
       </c>
       <c r="H155" s="12">
         <v>20</v>
@@ -17398,64 +17404,64 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A157" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B157" s="31" t="s">
+      <c r="B157" t="s">
         <v>73</v>
       </c>
-      <c r="C157" s="31" t="s">
+      <c r="C157" t="s">
         <v>60</v>
       </c>
-      <c r="D157" s="31">
+      <c r="D157">
         <v>1</v>
       </c>
-      <c r="E157" s="31">
-        <v>24</v>
-      </c>
-      <c r="F157" s="32"/>
-      <c r="H157" s="31">
+      <c r="E157">
+        <v>24</v>
+      </c>
+      <c r="F157" s="9"/>
+      <c r="H157">
         <v>95</v>
       </c>
-      <c r="I157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J157" s="31">
+      <c r="I157" t="s">
+        <v>28</v>
+      </c>
+      <c r="J157">
         <f t="shared" si="2"/>
         <v>55.5</v>
       </c>
-      <c r="K157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L157" s="31">
+      <c r="K157" t="s">
+        <v>28</v>
+      </c>
+      <c r="L157">
         <v>55</v>
       </c>
-      <c r="M157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N157" s="31">
+      <c r="M157" t="s">
+        <v>28</v>
+      </c>
+      <c r="N157">
         <v>58.5</v>
       </c>
-      <c r="O157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P157" s="31">
+      <c r="O157" t="s">
+        <v>28</v>
+      </c>
+      <c r="P157">
         <v>57.5</v>
       </c>
-      <c r="Q157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R157" s="31">
+      <c r="Q157" t="s">
+        <v>28</v>
+      </c>
+      <c r="R157">
         <v>51</v>
       </c>
-      <c r="S157" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T157" s="31">
+      <c r="S157" t="s">
+        <v>28</v>
+      </c>
+      <c r="T157">
         <v>58.5</v>
       </c>
-      <c r="V157" s="34">
+      <c r="V157" s="16">
         <v>0.44722222222222224</v>
       </c>
     </row>
@@ -17477,8 +17483,8 @@
       </c>
       <c r="F158" s="13"/>
       <c r="G158" s="12">
-        <f>SUM(H156:H158)</f>
-        <v>115</v>
+        <f>SUM(H156:H157)</f>
+        <v>110</v>
       </c>
       <c r="H158" s="12">
         <v>5</v>
@@ -17549,30 +17555,30 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="160" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A160" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B160" s="31" t="s">
+      <c r="B160" t="s">
         <v>73</v>
       </c>
-      <c r="C160" s="31" t="s">
+      <c r="C160" t="s">
         <v>60</v>
       </c>
-      <c r="D160" s="31">
+      <c r="D160">
         <v>1</v>
       </c>
-      <c r="E160" s="31">
+      <c r="E160">
         <v>48</v>
       </c>
-      <c r="F160" s="32"/>
-      <c r="H160" s="31">
+      <c r="F160" s="9"/>
+      <c r="H160">
         <v>20</v>
       </c>
-      <c r="I160" s="31" t="s">
+      <c r="I160" t="s">
         <v>50</v>
       </c>
-      <c r="J160" s="31" t="e">
+      <c r="J160" t="e">
         <f>AVERAGE(L160, N160, P160, R160)</f>
         <v>#DIV/0!</v>
       </c>
@@ -17595,8 +17601,8 @@
       </c>
       <c r="F161" s="13"/>
       <c r="G161" s="12">
-        <f>SUM(H159:H161)</f>
-        <v>120</v>
+        <f>SUM(H159:H160)</f>
+        <v>115</v>
       </c>
       <c r="H161" s="12">
         <v>5</v>
@@ -17643,46 +17649,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A163" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B163" s="31" t="s">
+      <c r="B163" t="s">
         <v>73</v>
       </c>
-      <c r="C163" s="31" t="s">
+      <c r="C163" t="s">
         <v>60</v>
       </c>
-      <c r="D163" s="31">
-        <v>2</v>
-      </c>
-      <c r="E163" s="31">
+      <c r="D163">
+        <v>2</v>
+      </c>
+      <c r="E163">
         <v>0.5</v>
       </c>
-      <c r="F163" s="32"/>
-      <c r="H163" s="31">
+      <c r="F163" s="9"/>
+      <c r="H163">
         <v>40</v>
       </c>
-      <c r="I163" s="31" t="s">
+      <c r="I163" t="s">
         <v>26</v>
       </c>
-      <c r="J163" s="31">
+      <c r="J163">
         <f t="shared" si="2"/>
         <v>77.75</v>
       </c>
-      <c r="L163" s="31">
+      <c r="L163">
         <v>85</v>
       </c>
-      <c r="N163" s="31">
+      <c r="N163">
         <v>76</v>
       </c>
-      <c r="P163" s="31">
+      <c r="P163">
         <v>72</v>
       </c>
-      <c r="R163" s="31">
+      <c r="R163">
         <v>78</v>
       </c>
-      <c r="T163" s="31">
+      <c r="T163">
         <v>85</v>
       </c>
     </row>
@@ -17704,8 +17710,8 @@
       </c>
       <c r="F164" s="13"/>
       <c r="G164" s="12">
-        <f>SUM(H162:H164)</f>
-        <v>100</v>
+        <f>SUM(H163:H164)</f>
+        <v>70</v>
       </c>
       <c r="H164" s="12">
         <v>30</v>
@@ -17800,67 +17806,67 @@
         <v>93</v>
       </c>
     </row>
-    <row r="166" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A166" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B166" s="31" t="s">
+      <c r="B166" t="s">
         <v>73</v>
       </c>
-      <c r="C166" s="31" t="s">
+      <c r="C166" t="s">
         <v>60</v>
       </c>
-      <c r="D166" s="31">
-        <v>2</v>
-      </c>
-      <c r="E166" s="31">
-        <v>2</v>
-      </c>
-      <c r="F166" s="32"/>
-      <c r="H166" s="31">
+      <c r="D166">
+        <v>2</v>
+      </c>
+      <c r="E166">
+        <v>2</v>
+      </c>
+      <c r="F166" s="9"/>
+      <c r="H166">
         <v>30</v>
       </c>
-      <c r="I166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J166" s="31">
+      <c r="I166" t="s">
+        <v>28</v>
+      </c>
+      <c r="J166">
         <f t="shared" si="2"/>
         <v>54.5</v>
       </c>
-      <c r="K166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L166" s="31">
+      <c r="K166" t="s">
+        <v>28</v>
+      </c>
+      <c r="L166">
         <v>68</v>
       </c>
-      <c r="M166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N166" s="31">
+      <c r="M166" t="s">
+        <v>28</v>
+      </c>
+      <c r="N166">
         <v>53</v>
       </c>
-      <c r="O166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P166" s="31">
+      <c r="O166" t="s">
+        <v>28</v>
+      </c>
+      <c r="P166">
         <v>51</v>
       </c>
-      <c r="Q166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R166" s="31">
+      <c r="Q166" t="s">
+        <v>28</v>
+      </c>
+      <c r="R166">
         <v>46</v>
       </c>
-      <c r="S166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T166" s="31">
+      <c r="S166" t="s">
+        <v>28</v>
+      </c>
+      <c r="T166">
         <v>68</v>
       </c>
-      <c r="U166" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="V166" s="34">
+      <c r="U166" t="s">
+        <v>28</v>
+      </c>
+      <c r="V166" s="16">
         <v>0.42916666666666664</v>
       </c>
     </row>
@@ -17882,8 +17888,8 @@
       </c>
       <c r="F167" s="13"/>
       <c r="G167" s="12">
-        <f>SUM(H165:H167)</f>
-        <v>100</v>
+        <f>SUM(H165:H166)</f>
+        <v>65</v>
       </c>
       <c r="H167" s="12">
         <v>35</v>
@@ -17930,67 +17936,67 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A169" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B169" s="31" t="s">
+      <c r="B169" t="s">
         <v>73</v>
       </c>
-      <c r="C169" s="31" t="s">
+      <c r="C169" t="s">
         <v>60</v>
       </c>
-      <c r="D169" s="31">
-        <v>2</v>
-      </c>
-      <c r="E169" s="31">
+      <c r="D169">
+        <v>2</v>
+      </c>
+      <c r="E169">
         <v>6</v>
       </c>
-      <c r="F169" s="32"/>
-      <c r="H169" s="31">
+      <c r="F169" s="9"/>
+      <c r="H169">
         <v>80</v>
       </c>
-      <c r="I169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J169" s="31">
+      <c r="I169" t="s">
+        <v>28</v>
+      </c>
+      <c r="J169">
         <f t="shared" si="2"/>
         <v>50</v>
       </c>
-      <c r="K169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L169" s="31">
+      <c r="K169" t="s">
+        <v>28</v>
+      </c>
+      <c r="L169">
         <v>51</v>
       </c>
-      <c r="M169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N169" s="31">
+      <c r="M169" t="s">
+        <v>28</v>
+      </c>
+      <c r="N169">
         <v>55</v>
       </c>
-      <c r="O169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P169" s="31">
+      <c r="O169" t="s">
+        <v>28</v>
+      </c>
+      <c r="P169">
         <v>49</v>
       </c>
-      <c r="Q169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R169" s="31">
+      <c r="Q169" t="s">
+        <v>28</v>
+      </c>
+      <c r="R169">
         <v>45</v>
       </c>
-      <c r="S169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T169" s="31">
+      <c r="S169" t="s">
+        <v>28</v>
+      </c>
+      <c r="T169">
         <v>55</v>
       </c>
-      <c r="U169" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="V169" s="34">
+      <c r="U169" t="s">
+        <v>28</v>
+      </c>
+      <c r="V169" s="16">
         <v>0.42708333333333331</v>
       </c>
     </row>
@@ -18012,8 +18018,8 @@
       </c>
       <c r="F170" s="13"/>
       <c r="G170" s="12">
-        <f>SUM(H168:H170)</f>
-        <v>105</v>
+        <f>SUM(H169:H170)</f>
+        <v>85</v>
       </c>
       <c r="H170" s="12">
         <v>5</v>
@@ -18060,67 +18066,67 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A172" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B172" s="31" t="s">
+      <c r="B172" t="s">
         <v>73</v>
       </c>
-      <c r="C172" s="31" t="s">
+      <c r="C172" t="s">
         <v>60</v>
       </c>
-      <c r="D172" s="31">
-        <v>2</v>
-      </c>
-      <c r="E172" s="31">
+      <c r="D172">
+        <v>2</v>
+      </c>
+      <c r="E172">
         <v>12</v>
       </c>
-      <c r="F172" s="32"/>
-      <c r="H172" s="31">
+      <c r="F172" s="9"/>
+      <c r="H172">
         <v>90</v>
       </c>
-      <c r="I172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="J172" s="31">
+      <c r="I172" t="s">
+        <v>28</v>
+      </c>
+      <c r="J172">
         <f t="shared" si="2"/>
         <v>52.125</v>
       </c>
-      <c r="K172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L172" s="31">
+      <c r="K172" t="s">
+        <v>28</v>
+      </c>
+      <c r="L172">
         <v>54.5</v>
       </c>
-      <c r="M172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="N172" s="31">
+      <c r="M172" t="s">
+        <v>28</v>
+      </c>
+      <c r="N172">
         <v>48</v>
       </c>
-      <c r="O172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="P172" s="31">
+      <c r="O172" t="s">
+        <v>28</v>
+      </c>
+      <c r="P172">
         <v>50</v>
       </c>
-      <c r="Q172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="R172" s="31">
+      <c r="Q172" t="s">
+        <v>28</v>
+      </c>
+      <c r="R172">
         <v>56</v>
       </c>
-      <c r="S172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="T172" s="31">
+      <c r="S172" t="s">
+        <v>28</v>
+      </c>
+      <c r="T172">
         <v>56</v>
       </c>
-      <c r="U172" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="V172" s="34">
+      <c r="U172" t="s">
+        <v>28</v>
+      </c>
+      <c r="V172" s="16">
         <v>0.42569444444444443</v>
       </c>
     </row>
@@ -18142,8 +18148,8 @@
       </c>
       <c r="F173" s="13"/>
       <c r="G173" s="12">
-        <f>SUM(H171:H173)</f>
-        <v>105</v>
+        <f>SUM(H171:H172)</f>
+        <v>95</v>
       </c>
       <c r="H173" s="12">
         <v>10</v>
@@ -18190,27 +18196,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:22" s="31" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A175" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B175" s="31" t="s">
+      <c r="B175" t="s">
         <v>73</v>
       </c>
-      <c r="C175" s="31" t="s">
+      <c r="C175" t="s">
         <v>60</v>
       </c>
-      <c r="D175" s="31">
-        <v>2</v>
-      </c>
-      <c r="E175" s="31">
+      <c r="D175">
+        <v>2</v>
+      </c>
+      <c r="E175">
         <v>18</v>
       </c>
-      <c r="F175" s="32"/>
-      <c r="H175" s="31">
+      <c r="F175" s="9"/>
+      <c r="H175">
         <v>10</v>
       </c>
-      <c r="I175" s="31" t="s">
+      <c r="I175" t="s">
         <v>50</v>
       </c>
     </row>
@@ -18232,8 +18238,8 @@
       </c>
       <c r="F176" s="13"/>
       <c r="G176" s="12">
-        <f>SUM(H174:H176)</f>
-        <v>100</v>
+        <f>SUM(H175:H176)</f>
+        <v>95</v>
       </c>
       <c r="H176" s="12">
         <v>85</v>
@@ -18331,8 +18337,8 @@
       </c>
       <c r="F178" s="13"/>
       <c r="G178" s="12">
-        <f>SUM(H177:H178)</f>
-        <v>100</v>
+        <f>SUM(H178)</f>
+        <v>95</v>
       </c>
       <c r="H178" s="12">
         <v>95</v>
@@ -18463,8 +18469,8 @@
       </c>
       <c r="F180" s="9"/>
       <c r="G180">
-        <f>SUM(H179:H180)</f>
-        <v>100</v>
+        <f>SUM(H179)</f>
+        <v>95</v>
       </c>
       <c r="H180">
         <v>5</v>

</xml_diff>

<commit_message>
Finishing veg data and re-running data and tiers
</commit_message>
<xml_diff>
--- a/data/veg (raw).xlsx
+++ b/data/veg (raw).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1534" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9B77853-A92A-4DEE-9188-320A5936DF49}"/>
+  <xr:revisionPtr revIDLastSave="1537" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AC81A4-10A1-49C0-9DD1-06EA6191C80B}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-22365" yWindow="4605" windowWidth="8865" windowHeight="5790" activeTab="1" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
   </bookViews>
   <sheets>
     <sheet name="winter" sheetId="1" r:id="rId1"/>
@@ -1818,8 +1818,8 @@
         <v>46074</v>
       </c>
       <c r="G7" s="12">
-        <f>SUM(H5:H7)</f>
-        <v>115</v>
+        <f>SUM(H5:H6)</f>
+        <v>70</v>
       </c>
       <c r="H7" s="12">
         <v>45</v>
@@ -10524,7 +10524,7 @@
         <v>31</v>
       </c>
       <c r="J5" s="4" t="e">
-        <f t="shared" ref="J4:J63" si="0">AVERAGE(L5, N5, P5, R5)</f>
+        <f t="shared" ref="J5:J63" si="0">AVERAGE(L5, N5, P5, R5)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U5" s="4" t="s">

</xml_diff>

<commit_message>
Finished pipeline! First go around on models!
</commit_message>
<xml_diff>
--- a/data/veg (raw).xlsx
+++ b/data/veg (raw).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1537" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AC81A4-10A1-49C0-9DD1-06EA6191C80B}"/>
+  <xr:revisionPtr revIDLastSave="1541" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{746DC602-3C60-4F1A-AAF5-2126A6B61390}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="1" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
   </bookViews>
   <sheets>
     <sheet name="winter" sheetId="1" r:id="rId1"/>
@@ -14508,7 +14508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3" t="s">
         <v>69</v>
       </c>
@@ -14524,7 +14524,9 @@
       <c r="E92" s="4">
         <v>0.5</v>
       </c>
-      <c r="F92" s="5"/>
+      <c r="F92" s="5">
+        <v>46183</v>
+      </c>
       <c r="H92" s="4">
         <v>75</v>
       </c>
@@ -14532,7 +14534,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="93" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A93" s="27" t="s">
         <v>69</v>
       </c>
@@ -14548,7 +14550,9 @@
       <c r="E93" s="10">
         <v>0.5</v>
       </c>
-      <c r="F93" s="28"/>
+      <c r="F93" s="5">
+        <v>46183</v>
+      </c>
       <c r="H93" s="10">
         <v>80</v>
       </c>
@@ -14594,7 +14598,9 @@
       <c r="E94" s="14">
         <v>0.5</v>
       </c>
-      <c r="F94" s="33"/>
+      <c r="F94" s="5">
+        <v>46183</v>
+      </c>
       <c r="G94" s="14">
         <f>SUM(H92:H94)</f>
         <v>160</v>
@@ -14637,7 +14643,7 @@
         <v>0.60763888888888884</v>
       </c>
     </row>
-    <row r="95" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A95" s="3" t="s">
         <v>69</v>
       </c>
@@ -14653,7 +14659,9 @@
       <c r="E95" s="4">
         <v>2</v>
       </c>
-      <c r="F95" s="5"/>
+      <c r="F95" s="5">
+        <v>46183</v>
+      </c>
       <c r="H95" s="4">
         <v>50</v>
       </c>
@@ -14664,7 +14672,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="96" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A96" s="27" t="s">
         <v>69</v>
       </c>
@@ -14680,7 +14688,9 @@
       <c r="E96" s="10">
         <v>2</v>
       </c>
-      <c r="F96" s="28"/>
+      <c r="F96" s="5">
+        <v>46183</v>
+      </c>
       <c r="H96" s="10">
         <v>10</v>
       </c>
@@ -14723,7 +14733,9 @@
       <c r="E97" s="14">
         <v>2</v>
       </c>
-      <c r="F97" s="33"/>
+      <c r="F97" s="5">
+        <v>46183</v>
+      </c>
       <c r="G97" s="14">
         <f>SUM(H95:H97)</f>
         <v>135</v>
@@ -14760,7 +14772,7 @@
         <v>0.60069444444444442</v>
       </c>
     </row>
-    <row r="98" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A98" s="29" t="s">
         <v>69</v>
       </c>
@@ -14776,7 +14788,9 @@
       <c r="E98" s="6">
         <v>6</v>
       </c>
-      <c r="F98" s="30"/>
+      <c r="F98" s="5">
+        <v>46183</v>
+      </c>
       <c r="H98" s="6">
         <v>95</v>
       </c>
@@ -14822,7 +14836,9 @@
       <c r="E99" s="12">
         <v>6</v>
       </c>
-      <c r="F99" s="13"/>
+      <c r="F99" s="5">
+        <v>46183</v>
+      </c>
       <c r="G99" s="12">
         <f>SUM(H98)</f>
         <v>95</v>
@@ -14844,7 +14860,7 @@
         <v>0.59513888888888888</v>
       </c>
     </row>
-    <row r="100" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="29" t="s">
         <v>69</v>
       </c>
@@ -14860,7 +14876,9 @@
       <c r="E100" s="6">
         <v>12</v>
       </c>
-      <c r="F100" s="30"/>
+      <c r="F100" s="5">
+        <v>46183</v>
+      </c>
       <c r="H100" s="6">
         <v>60</v>
       </c>
@@ -14908,7 +14926,7 @@
         <v>0.58611111111111114</v>
       </c>
     </row>
-    <row r="101" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="27" t="s">
         <v>69</v>
       </c>
@@ -14924,7 +14942,9 @@
       <c r="E101" s="10">
         <v>12</v>
       </c>
-      <c r="F101" s="28"/>
+      <c r="F101" s="5">
+        <v>46183</v>
+      </c>
       <c r="H101" s="10">
         <v>20</v>
       </c>
@@ -14973,7 +14993,9 @@
       <c r="E102" s="12">
         <v>12</v>
       </c>
-      <c r="F102" s="13"/>
+      <c r="F102" s="5">
+        <v>46183</v>
+      </c>
       <c r="G102" s="12">
         <f>SUM(H100:H101)</f>
         <v>80</v>
@@ -14992,7 +15014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="29" t="s">
         <v>69</v>
       </c>
@@ -15008,7 +15030,9 @@
       <c r="E103" s="6">
         <v>18</v>
       </c>
-      <c r="F103" s="30"/>
+      <c r="F103" s="5">
+        <v>46183</v>
+      </c>
       <c r="H103" s="6">
         <v>35</v>
       </c>
@@ -15056,7 +15080,7 @@
         <v>0.5756944444444444</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="8" t="s">
         <v>69</v>
       </c>
@@ -15072,7 +15096,9 @@
       <c r="E104">
         <v>18</v>
       </c>
-      <c r="F104" s="9"/>
+      <c r="F104" s="5">
+        <v>46183</v>
+      </c>
       <c r="H104">
         <v>10</v>
       </c>
@@ -15087,7 +15113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A105" s="27" t="s">
         <v>69</v>
       </c>
@@ -15103,7 +15129,9 @@
       <c r="E105" s="10">
         <v>18</v>
       </c>
-      <c r="F105" s="28"/>
+      <c r="F105" s="5">
+        <v>46183</v>
+      </c>
       <c r="H105" s="10">
         <v>45</v>
       </c>
@@ -15152,7 +15180,9 @@
       <c r="E106" s="12">
         <v>18</v>
       </c>
-      <c r="F106" s="13"/>
+      <c r="F106" s="5">
+        <v>46183</v>
+      </c>
       <c r="G106" s="12">
         <f>SUM(H103:H105)</f>
         <v>90</v>
@@ -15174,7 +15204,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="107" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A107" s="29" t="s">
         <v>69</v>
       </c>
@@ -15190,7 +15220,9 @@
       <c r="E107" s="6">
         <v>24</v>
       </c>
-      <c r="F107" s="30"/>
+      <c r="F107" s="5">
+        <v>46183</v>
+      </c>
       <c r="H107" s="6">
         <v>15</v>
       </c>
@@ -15238,7 +15270,7 @@
         <v>0.5625</v>
       </c>
     </row>
-    <row r="108" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="27" t="s">
         <v>69</v>
       </c>
@@ -15254,7 +15286,9 @@
       <c r="E108" s="10">
         <v>24</v>
       </c>
-      <c r="F108" s="28"/>
+      <c r="F108" s="5">
+        <v>46183</v>
+      </c>
       <c r="H108" s="10">
         <v>80</v>
       </c>
@@ -15287,7 +15321,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="109" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A109" s="27" t="s">
         <v>69</v>
       </c>
@@ -15303,7 +15337,9 @@
       <c r="E109" s="10">
         <v>24</v>
       </c>
-      <c r="F109" s="28"/>
+      <c r="F109" s="5">
+        <v>46183</v>
+      </c>
       <c r="H109" s="10">
         <v>20</v>
       </c>
@@ -15349,7 +15385,9 @@
       <c r="E110" s="12">
         <v>24</v>
       </c>
-      <c r="F110" s="13"/>
+      <c r="F110" s="5">
+        <v>46183</v>
+      </c>
       <c r="G110" s="12">
         <f>SUM(H107:H110)</f>
         <v>120</v>
@@ -15368,7 +15406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A111" s="3" t="s">
         <v>69</v>
       </c>
@@ -15384,7 +15422,9 @@
       <c r="E111" s="4">
         <v>48</v>
       </c>
-      <c r="F111" s="5"/>
+      <c r="F111" s="5">
+        <v>46183</v>
+      </c>
       <c r="H111" s="4">
         <v>5</v>
       </c>
@@ -15399,7 +15439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A112" s="27" t="s">
         <v>69</v>
       </c>
@@ -15415,7 +15455,9 @@
       <c r="E112" s="10">
         <v>48</v>
       </c>
-      <c r="F112" s="28"/>
+      <c r="F112" s="5">
+        <v>46183</v>
+      </c>
       <c r="H112" s="10">
         <v>90</v>
       </c>
@@ -15464,7 +15506,9 @@
       <c r="E113" s="14">
         <v>48</v>
       </c>
-      <c r="F113" s="33"/>
+      <c r="F113" s="5">
+        <v>46183</v>
+      </c>
       <c r="G113" s="14">
         <f>SUM(H112:H113)</f>
         <v>95</v>
@@ -15498,7 +15542,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A114" s="29" t="s">
         <v>69</v>
       </c>
@@ -15514,7 +15558,9 @@
       <c r="E114" s="6">
         <v>0.5</v>
       </c>
-      <c r="F114" s="30"/>
+      <c r="F114" s="5">
+        <v>46183</v>
+      </c>
       <c r="H114" s="6">
         <v>20</v>
       </c>
@@ -15562,7 +15608,7 @@
         <v>0.62708333333333333</v>
       </c>
     </row>
-    <row r="115" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A115" s="27" t="s">
         <v>69</v>
       </c>
@@ -15578,7 +15624,9 @@
       <c r="E115" s="10">
         <v>0.5</v>
       </c>
-      <c r="F115" s="28"/>
+      <c r="F115" s="5">
+        <v>46183</v>
+      </c>
       <c r="H115" s="10">
         <v>75</v>
       </c>
@@ -15608,7 +15656,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="8" t="s">
         <v>69</v>
       </c>
@@ -15624,7 +15672,9 @@
       <c r="E116">
         <v>0.5</v>
       </c>
-      <c r="F116" s="9"/>
+      <c r="F116" s="5">
+        <v>46183</v>
+      </c>
       <c r="H116">
         <v>15</v>
       </c>
@@ -15655,7 +15705,9 @@
       <c r="E117" s="12">
         <v>0.5</v>
       </c>
-      <c r="F117" s="13"/>
+      <c r="F117" s="5">
+        <v>46183</v>
+      </c>
       <c r="G117" s="12">
         <f>SUM(H114:H116)</f>
         <v>110</v>
@@ -15674,7 +15726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="29" t="s">
         <v>69</v>
       </c>
@@ -15690,7 +15742,9 @@
       <c r="E118" s="6">
         <v>2</v>
       </c>
-      <c r="F118" s="30"/>
+      <c r="F118" s="5">
+        <v>46183</v>
+      </c>
       <c r="H118" s="6">
         <v>20</v>
       </c>
@@ -15738,7 +15792,7 @@
         <v>0.63541666666666663</v>
       </c>
     </row>
-    <row r="119" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A119" s="27" t="s">
         <v>69</v>
       </c>
@@ -15754,7 +15808,9 @@
       <c r="E119" s="10">
         <v>2</v>
       </c>
-      <c r="F119" s="28"/>
+      <c r="F119" s="5">
+        <v>46183</v>
+      </c>
       <c r="H119" s="10">
         <v>75</v>
       </c>
@@ -15784,7 +15840,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A120" s="8" t="s">
         <v>69</v>
       </c>
@@ -15800,7 +15856,9 @@
       <c r="E120">
         <v>2</v>
       </c>
-      <c r="F120" s="9"/>
+      <c r="F120" s="5">
+        <v>46183</v>
+      </c>
       <c r="H120">
         <v>65</v>
       </c>
@@ -15846,7 +15904,9 @@
       <c r="E121" s="12">
         <v>2</v>
       </c>
-      <c r="F121" s="13"/>
+      <c r="F121" s="5">
+        <v>46183</v>
+      </c>
       <c r="G121" s="12">
         <f>SUM(H118:H120)</f>
         <v>160</v>
@@ -15865,7 +15925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A122" s="29" t="s">
         <v>69</v>
       </c>
@@ -15881,7 +15941,9 @@
       <c r="E122" s="6">
         <v>6</v>
       </c>
-      <c r="F122" s="30"/>
+      <c r="F122" s="5">
+        <v>46183</v>
+      </c>
       <c r="H122" s="6">
         <v>40</v>
       </c>
@@ -15929,7 +15991,7 @@
         <v>0.6430555555555556</v>
       </c>
     </row>
-    <row r="123" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A123" s="27" t="s">
         <v>69</v>
       </c>
@@ -15945,7 +16007,9 @@
       <c r="E123" s="10">
         <v>6</v>
       </c>
-      <c r="F123" s="28"/>
+      <c r="F123" s="5">
+        <v>46183</v>
+      </c>
       <c r="H123" s="10">
         <v>50</v>
       </c>
@@ -15975,7 +16039,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A124" s="8" t="s">
         <v>69</v>
       </c>
@@ -15991,7 +16055,9 @@
       <c r="E124">
         <v>6</v>
       </c>
-      <c r="F124" s="9"/>
+      <c r="F124" s="5">
+        <v>46183</v>
+      </c>
       <c r="H124">
         <v>30</v>
       </c>
@@ -16006,7 +16072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A125" s="27" t="s">
         <v>69</v>
       </c>
@@ -16022,7 +16088,9 @@
       <c r="E125" s="10">
         <v>6</v>
       </c>
-      <c r="F125" s="28"/>
+      <c r="F125" s="5">
+        <v>46183</v>
+      </c>
       <c r="H125" s="10">
         <v>10</v>
       </c>
@@ -16068,7 +16136,9 @@
       <c r="E126" s="12">
         <v>6</v>
       </c>
-      <c r="F126" s="13"/>
+      <c r="F126" s="5">
+        <v>46183</v>
+      </c>
       <c r="G126" s="12">
         <f>SUM(H122:H125)</f>
         <v>130</v>
@@ -16087,7 +16157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A127" s="3" t="s">
         <v>69</v>
       </c>
@@ -16103,7 +16173,9 @@
       <c r="E127" s="4">
         <v>12</v>
       </c>
-      <c r="F127" s="5"/>
+      <c r="F127" s="5">
+        <v>46183</v>
+      </c>
       <c r="H127" s="4">
         <v>10</v>
       </c>
@@ -16121,7 +16193,7 @@
         <v>0.65208333333333335</v>
       </c>
     </row>
-    <row r="128" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="27" t="s">
         <v>69</v>
       </c>
@@ -16137,7 +16209,9 @@
       <c r="E128" s="10">
         <v>12</v>
       </c>
-      <c r="F128" s="28"/>
+      <c r="F128" s="5">
+        <v>46183</v>
+      </c>
       <c r="H128" s="10">
         <v>35</v>
       </c>
@@ -16182,7 +16256,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A129" s="27" t="s">
         <v>69</v>
       </c>
@@ -16198,7 +16272,9 @@
       <c r="E129" s="10">
         <v>12</v>
       </c>
-      <c r="F129" s="28"/>
+      <c r="F129" s="5">
+        <v>46183</v>
+      </c>
       <c r="H129" s="10">
         <v>55</v>
       </c>
@@ -16228,7 +16304,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A130" s="8" t="s">
         <v>69</v>
       </c>
@@ -16244,7 +16320,9 @@
       <c r="E130">
         <v>12</v>
       </c>
-      <c r="F130" s="9"/>
+      <c r="F130" s="5">
+        <v>46183</v>
+      </c>
       <c r="H130">
         <v>10</v>
       </c>
@@ -16278,7 +16356,9 @@
       <c r="E131" s="14">
         <v>12</v>
       </c>
-      <c r="F131" s="33"/>
+      <c r="F131" s="5">
+        <v>46183</v>
+      </c>
       <c r="G131" s="14">
         <f>SUM(H128:H131)</f>
         <v>115</v>
@@ -16312,7 +16392,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="132" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A132" s="3" t="s">
         <v>69</v>
       </c>
@@ -16328,7 +16408,9 @@
       <c r="E132" s="4">
         <v>18</v>
       </c>
-      <c r="F132" s="5"/>
+      <c r="F132" s="5">
+        <v>46183</v>
+      </c>
       <c r="H132" s="4">
         <v>15</v>
       </c>
@@ -16346,7 +16428,7 @@
         <v>0.66388888888888886</v>
       </c>
     </row>
-    <row r="133" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A133" s="27" t="s">
         <v>69</v>
       </c>
@@ -16362,7 +16444,9 @@
       <c r="E133" s="10">
         <v>18</v>
       </c>
-      <c r="F133" s="28"/>
+      <c r="F133" s="5">
+        <v>46183</v>
+      </c>
       <c r="H133" s="10">
         <v>25</v>
       </c>
@@ -16407,7 +16491,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="134" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A134" s="27" t="s">
         <v>69</v>
       </c>
@@ -16423,7 +16507,9 @@
       <c r="E134" s="10">
         <v>18</v>
       </c>
-      <c r="F134" s="28"/>
+      <c r="F134" s="5">
+        <v>46183</v>
+      </c>
       <c r="H134" s="10">
         <v>35</v>
       </c>
@@ -16469,7 +16555,9 @@
       <c r="E135" s="14">
         <v>18</v>
       </c>
-      <c r="F135" s="33"/>
+      <c r="F135" s="5">
+        <v>46183</v>
+      </c>
       <c r="G135" s="14">
         <f>SUM(H133:H135)</f>
         <v>105</v>
@@ -16500,7 +16588,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A136" s="3" t="s">
         <v>69</v>
       </c>
@@ -16516,7 +16604,9 @@
       <c r="E136" s="4">
         <v>24</v>
       </c>
-      <c r="F136" s="5"/>
+      <c r="F136" s="5">
+        <v>46183</v>
+      </c>
       <c r="H136" s="4">
         <v>5</v>
       </c>
@@ -16531,7 +16621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A137" s="27" t="s">
         <v>69</v>
       </c>
@@ -16547,7 +16637,9 @@
       <c r="E137" s="10">
         <v>24</v>
       </c>
-      <c r="F137" s="28"/>
+      <c r="F137" s="5">
+        <v>46183</v>
+      </c>
       <c r="H137" s="10">
         <v>20</v>
       </c>
@@ -16580,7 +16672,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="138" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="27" t="s">
         <v>69</v>
       </c>
@@ -16596,7 +16688,9 @@
       <c r="E138" s="10">
         <v>24</v>
       </c>
-      <c r="F138" s="28"/>
+      <c r="F138" s="5">
+        <v>46183</v>
+      </c>
       <c r="H138" s="10">
         <v>25</v>
       </c>
@@ -16644,7 +16738,7 @@
         <v>0.6743055555555556</v>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A139" s="8" t="s">
         <v>69</v>
       </c>
@@ -16660,7 +16754,9 @@
       <c r="E139">
         <v>24</v>
       </c>
-      <c r="F139" s="9"/>
+      <c r="F139" s="5">
+        <v>46183</v>
+      </c>
       <c r="H139">
         <v>10</v>
       </c>
@@ -16691,7 +16787,9 @@
       <c r="E140" s="14">
         <v>24</v>
       </c>
-      <c r="F140" s="33"/>
+      <c r="F140" s="5">
+        <v>46183</v>
+      </c>
       <c r="G140" s="14">
         <f>SUM(H137:H140)</f>
         <v>120</v>
@@ -16725,7 +16823,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="141" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="3" t="s">
         <v>69</v>
       </c>
@@ -16741,7 +16839,9 @@
       <c r="E141" s="4">
         <v>48</v>
       </c>
-      <c r="F141" s="5"/>
+      <c r="F141" s="5">
+        <v>46183</v>
+      </c>
       <c r="H141" s="4">
         <v>5</v>
       </c>
@@ -16759,7 +16859,7 @@
         <v>0.68541666666666667</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="8" t="s">
         <v>69</v>
       </c>
@@ -16775,7 +16875,9 @@
       <c r="E142">
         <v>48</v>
       </c>
-      <c r="F142" s="9"/>
+      <c r="F142" s="5">
+        <v>46183</v>
+      </c>
       <c r="H142">
         <v>35</v>
       </c>
@@ -16793,7 +16895,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="143" spans="1:23" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="27" t="s">
         <v>69</v>
       </c>
@@ -16809,7 +16911,9 @@
       <c r="E143" s="10">
         <v>48</v>
       </c>
-      <c r="F143" s="28"/>
+      <c r="F143" s="5">
+        <v>46183</v>
+      </c>
       <c r="H143" s="10">
         <v>90</v>
       </c>
@@ -16855,7 +16959,9 @@
       <c r="E144" s="14">
         <v>48</v>
       </c>
-      <c r="F144" s="33"/>
+      <c r="F144" s="5">
+        <v>46183</v>
+      </c>
       <c r="G144" s="14">
         <f>SUM(H142:H144)</f>
         <v>130</v>
@@ -16889,7 +16995,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="145" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A145" s="29" t="s">
         <v>69</v>
       </c>
@@ -16905,7 +17011,9 @@
       <c r="E145" s="6">
         <v>0.5</v>
       </c>
-      <c r="F145" s="30"/>
+      <c r="F145" s="30">
+        <v>46185</v>
+      </c>
       <c r="H145" s="6">
         <v>35</v>
       </c>
@@ -16953,7 +17061,7 @@
         <v>0.43541666666666667</v>
       </c>
     </row>
-    <row r="146" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A146" s="27" t="s">
         <v>69</v>
       </c>
@@ -16969,7 +17077,9 @@
       <c r="E146" s="10">
         <v>0.5</v>
       </c>
-      <c r="F146" s="28"/>
+      <c r="F146" s="30">
+        <v>46185</v>
+      </c>
       <c r="H146" s="10">
         <v>35</v>
       </c>
@@ -17012,7 +17122,9 @@
       <c r="E147" s="12">
         <v>0.5</v>
       </c>
-      <c r="F147" s="13"/>
+      <c r="F147" s="30">
+        <v>46185</v>
+      </c>
       <c r="G147" s="12">
         <f>SUM(H145:H146)</f>
         <v>70</v>
@@ -17031,7 +17143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A148" s="29" t="s">
         <v>69</v>
       </c>
@@ -17047,7 +17159,9 @@
       <c r="E148" s="6">
         <v>2</v>
       </c>
-      <c r="F148" s="30"/>
+      <c r="F148" s="30">
+        <v>46185</v>
+      </c>
       <c r="H148" s="6">
         <v>75</v>
       </c>
@@ -17111,7 +17225,9 @@
       <c r="E149" s="12">
         <v>2</v>
       </c>
-      <c r="F149" s="13"/>
+      <c r="F149" s="30">
+        <v>46185</v>
+      </c>
       <c r="G149" s="12">
         <f>SUM(H148)</f>
         <v>75</v>
@@ -17130,7 +17246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A150" s="3" t="s">
         <v>69</v>
       </c>
@@ -17146,7 +17262,9 @@
       <c r="E150" s="4">
         <v>6</v>
       </c>
-      <c r="F150" s="5"/>
+      <c r="F150" s="30">
+        <v>46185</v>
+      </c>
       <c r="H150" s="4">
         <v>40</v>
       </c>
@@ -17177,7 +17295,9 @@
       <c r="E151" s="14">
         <v>6</v>
       </c>
-      <c r="F151" s="33"/>
+      <c r="F151" s="30">
+        <v>46185</v>
+      </c>
       <c r="G151" s="14">
         <f>SUM(H151)</f>
         <v>60</v>
@@ -17229,7 +17349,7 @@
         <v>0.44027777777777777</v>
       </c>
     </row>
-    <row r="152" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A152" s="29" t="s">
         <v>69</v>
       </c>
@@ -17245,7 +17365,9 @@
       <c r="E152" s="6">
         <v>12</v>
       </c>
-      <c r="F152" s="30"/>
+      <c r="F152" s="30">
+        <v>46185</v>
+      </c>
       <c r="H152" s="6">
         <v>65</v>
       </c>
@@ -17309,7 +17431,9 @@
       <c r="E153" s="12">
         <v>12</v>
       </c>
-      <c r="F153" s="13"/>
+      <c r="F153" s="30">
+        <v>46185</v>
+      </c>
       <c r="G153" s="12">
         <f>SUM(H152)</f>
         <v>65</v>
@@ -17328,7 +17452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A154" s="29" t="s">
         <v>69</v>
       </c>
@@ -17344,7 +17468,9 @@
       <c r="E154" s="6">
         <v>18</v>
       </c>
-      <c r="F154" s="30"/>
+      <c r="F154" s="30">
+        <v>46185</v>
+      </c>
       <c r="H154" s="6">
         <v>80</v>
       </c>
@@ -17408,7 +17534,9 @@
       <c r="E155" s="12">
         <v>18</v>
       </c>
-      <c r="F155" s="13"/>
+      <c r="F155" s="30">
+        <v>46185</v>
+      </c>
       <c r="G155" s="12">
         <f>SUM(H154)</f>
         <v>80</v>
@@ -17427,7 +17555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A156" s="3" t="s">
         <v>69</v>
       </c>
@@ -17443,7 +17571,9 @@
       <c r="E156" s="4">
         <v>24</v>
       </c>
-      <c r="F156" s="5"/>
+      <c r="F156" s="30">
+        <v>46185</v>
+      </c>
       <c r="H156" s="4">
         <v>15</v>
       </c>
@@ -17458,7 +17588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A157" s="27" t="s">
         <v>69</v>
       </c>
@@ -17474,7 +17604,9 @@
       <c r="E157" s="10">
         <v>24</v>
       </c>
-      <c r="F157" s="28"/>
+      <c r="F157" s="30">
+        <v>46185</v>
+      </c>
       <c r="H157" s="10">
         <v>95</v>
       </c>
@@ -17535,7 +17667,9 @@
       <c r="E158" s="12">
         <v>24</v>
       </c>
-      <c r="F158" s="13"/>
+      <c r="F158" s="30">
+        <v>46185</v>
+      </c>
       <c r="G158" s="12">
         <f>SUM(H156:H157)</f>
         <v>110</v>
@@ -17554,7 +17688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="29" t="s">
         <v>69</v>
       </c>
@@ -17570,7 +17704,9 @@
       <c r="E159" s="6">
         <v>48</v>
       </c>
-      <c r="F159" s="30"/>
+      <c r="F159" s="30">
+        <v>46185</v>
+      </c>
       <c r="H159" s="6">
         <v>95</v>
       </c>
@@ -17609,7 +17745,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="160" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="8" t="s">
         <v>69</v>
       </c>
@@ -17625,7 +17761,9 @@
       <c r="E160">
         <v>48</v>
       </c>
-      <c r="F160" s="9"/>
+      <c r="F160" s="30">
+        <v>46185</v>
+      </c>
       <c r="H160">
         <v>20</v>
       </c>
@@ -17653,7 +17791,9 @@
       <c r="E161" s="12">
         <v>48</v>
       </c>
-      <c r="F161" s="13"/>
+      <c r="F161" s="30">
+        <v>46185</v>
+      </c>
       <c r="G161" s="12">
         <f>SUM(H159:H160)</f>
         <v>115</v>
@@ -17672,7 +17812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="3" t="s">
         <v>69</v>
       </c>
@@ -17688,7 +17828,9 @@
       <c r="E162" s="4">
         <v>0.5</v>
       </c>
-      <c r="F162" s="5"/>
+      <c r="F162" s="30">
+        <v>46185</v>
+      </c>
       <c r="H162" s="4">
         <v>30</v>
       </c>
@@ -17703,7 +17845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A163" s="27" t="s">
         <v>69</v>
       </c>
@@ -17719,7 +17861,9 @@
       <c r="E163" s="10">
         <v>0.5</v>
       </c>
-      <c r="F163" s="28"/>
+      <c r="F163" s="30">
+        <v>46185</v>
+      </c>
       <c r="H163" s="10">
         <v>40</v>
       </c>
@@ -17762,7 +17906,9 @@
       <c r="E164" s="14">
         <v>0.5</v>
       </c>
-      <c r="F164" s="33"/>
+      <c r="F164" s="30">
+        <v>46185</v>
+      </c>
       <c r="G164" s="14">
         <f>SUM(H163:H164)</f>
         <v>70</v>
@@ -17814,7 +17960,7 @@
         <v>0.43194444444444446</v>
       </c>
     </row>
-    <row r="165" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:22" s="6" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="29" t="s">
         <v>69</v>
       </c>
@@ -17830,7 +17976,9 @@
       <c r="E165" s="6">
         <v>2</v>
       </c>
-      <c r="F165" s="30"/>
+      <c r="F165" s="30">
+        <v>46185</v>
+      </c>
       <c r="H165" s="6">
         <v>35</v>
       </c>
@@ -17860,7 +18008,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="166" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A166" s="27" t="s">
         <v>69</v>
       </c>
@@ -17876,7 +18024,9 @@
       <c r="E166" s="10">
         <v>2</v>
       </c>
-      <c r="F166" s="28"/>
+      <c r="F166" s="30">
+        <v>46185</v>
+      </c>
       <c r="H166" s="10">
         <v>30</v>
       </c>
@@ -17940,7 +18090,9 @@
       <c r="E167" s="12">
         <v>2</v>
       </c>
-      <c r="F167" s="13"/>
+      <c r="F167" s="30">
+        <v>46185</v>
+      </c>
       <c r="G167" s="12">
         <f>SUM(H165:H166)</f>
         <v>65</v>
@@ -17959,7 +18111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="3" t="s">
         <v>69</v>
       </c>
@@ -17975,7 +18127,9 @@
       <c r="E168" s="4">
         <v>6</v>
       </c>
-      <c r="F168" s="5"/>
+      <c r="F168" s="30">
+        <v>46185</v>
+      </c>
       <c r="H168" s="4">
         <v>20</v>
       </c>
@@ -17990,7 +18144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A169" s="27" t="s">
         <v>69</v>
       </c>
@@ -18006,7 +18160,9 @@
       <c r="E169" s="10">
         <v>6</v>
       </c>
-      <c r="F169" s="28"/>
+      <c r="F169" s="30">
+        <v>46185</v>
+      </c>
       <c r="H169" s="10">
         <v>80</v>
       </c>
@@ -18070,7 +18226,9 @@
       <c r="E170" s="12">
         <v>6</v>
       </c>
-      <c r="F170" s="13"/>
+      <c r="F170" s="30">
+        <v>46185</v>
+      </c>
       <c r="G170" s="12">
         <f>SUM(H169:H170)</f>
         <v>85</v>
@@ -18089,7 +18247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="3" t="s">
         <v>69</v>
       </c>
@@ -18105,7 +18263,9 @@
       <c r="E171" s="4">
         <v>12</v>
       </c>
-      <c r="F171" s="5"/>
+      <c r="F171" s="30">
+        <v>46185</v>
+      </c>
       <c r="H171" s="4">
         <v>5</v>
       </c>
@@ -18120,7 +18280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="27" t="s">
         <v>69</v>
       </c>
@@ -18136,7 +18296,9 @@
       <c r="E172" s="10">
         <v>12</v>
       </c>
-      <c r="F172" s="28"/>
+      <c r="F172" s="30">
+        <v>46185</v>
+      </c>
       <c r="H172" s="10">
         <v>90</v>
       </c>
@@ -18200,7 +18362,9 @@
       <c r="E173" s="12">
         <v>12</v>
       </c>
-      <c r="F173" s="13"/>
+      <c r="F173" s="30">
+        <v>46185</v>
+      </c>
       <c r="G173" s="12">
         <f>SUM(H171:H172)</f>
         <v>95</v>
@@ -18219,7 +18383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A174" s="3" t="s">
         <v>69</v>
       </c>
@@ -18235,7 +18399,9 @@
       <c r="E174" s="4">
         <v>18</v>
       </c>
-      <c r="F174" s="5"/>
+      <c r="F174" s="30">
+        <v>46185</v>
+      </c>
       <c r="H174" s="4">
         <v>5</v>
       </c>
@@ -18250,7 +18416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A175" s="8" t="s">
         <v>69</v>
       </c>
@@ -18266,7 +18432,9 @@
       <c r="E175">
         <v>18</v>
       </c>
-      <c r="F175" s="9"/>
+      <c r="F175" s="30">
+        <v>46185</v>
+      </c>
       <c r="H175">
         <v>10</v>
       </c>
@@ -18290,7 +18458,9 @@
       <c r="E176" s="14">
         <v>18</v>
       </c>
-      <c r="F176" s="33"/>
+      <c r="F176" s="30">
+        <v>46185</v>
+      </c>
       <c r="G176" s="14">
         <f>SUM(H175:H176)</f>
         <v>95</v>
@@ -18342,7 +18512,7 @@
         <v>0.4236111111111111</v>
       </c>
     </row>
-    <row r="177" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:22" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="3" t="s">
         <v>69</v>
       </c>
@@ -18358,7 +18528,9 @@
       <c r="E177" s="4">
         <v>24</v>
       </c>
-      <c r="F177" s="5"/>
+      <c r="F177" s="30">
+        <v>46185</v>
+      </c>
       <c r="H177" s="4">
         <v>5</v>
       </c>
@@ -18389,7 +18561,9 @@
       <c r="E178" s="14">
         <v>24</v>
       </c>
-      <c r="F178" s="33"/>
+      <c r="F178" s="30">
+        <v>46185</v>
+      </c>
       <c r="G178" s="14">
         <f>SUM(H178)</f>
         <v>95</v>
@@ -18441,7 +18615,7 @@
         <v>0.41944444444444445</v>
       </c>
     </row>
-    <row r="179" spans="1:22" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:22" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="10" t="s">
         <v>69</v>
       </c>
@@ -18457,7 +18631,9 @@
       <c r="E179" s="10">
         <v>48</v>
       </c>
-      <c r="F179" s="28"/>
+      <c r="F179" s="30">
+        <v>46185</v>
+      </c>
       <c r="H179" s="10">
         <v>95</v>
       </c>
@@ -18521,7 +18697,9 @@
       <c r="E180">
         <v>48</v>
       </c>
-      <c r="F180" s="9"/>
+      <c r="F180" s="30">
+        <v>46185</v>
+      </c>
       <c r="G180">
         <f>SUM(H179)</f>
         <v>95</v>

</xml_diff>

<commit_message>
Edit and fine tune first draft of results
</commit_message>
<xml_diff>
--- a/data/veg (raw).xlsx
+++ b/data/veg (raw).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1541" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{746DC602-3C60-4F1A-AAF5-2126A6B61390}"/>
+  <xr:revisionPtr revIDLastSave="1545" documentId="8_{92FB2599-59FD-4CA2-946A-D08153E8274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2567147-C3A5-4908-AC8B-868A1D2A0612}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="1" xr2:uid="{4ED2C885-2CC1-498F-A981-739A00DDA370}"/>
   </bookViews>
@@ -1451,18 +1451,18 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="12.77734375" customWidth="1"/>
     <col min="10" max="10" width="11.6640625" customWidth="1"/>
     <col min="11" max="11" width="9.109375" customWidth="1"/>
-    <col min="12" max="12" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="8.77734375" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="14.5546875" customWidth="1"/>
     <col min="22" max="22" width="11.77734375" customWidth="1"/>
   </cols>
@@ -10245,18 +10245,19 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.77734375" customWidth="1"/>
     <col min="10" max="10" width="11.6640625" customWidth="1"/>
-    <col min="11" max="11" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="8.77734375" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="14.5546875" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="11.77734375" customWidth="1"/>
   </cols>

</xml_diff>